<commit_message>
Redesign Audit Checklist for readability
Wider columns, taller rows, and full-width colored section-header
bands between each of the 5 categories. Larger overall-% box and
performance-band cell at the bottom. Auto-scoring unchanged.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,55 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000B5555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -132,8 +179,18 @@
         <fgColor rgb="00F8C9C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B5555"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -160,11 +217,88 @@
       <right/>
       <bottom/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -233,6 +367,54 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,580 +812,626 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Clinical Documentation Audit — Checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>One chart · one page · tick each element ✓ Met · △ Partial · ✗ Not Met · N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Clinical Documentation Audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>One chart per sheet · tick each item · scoring &amp; rating are automatic</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>Provider:</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Date of Service:</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>How to use
-• Pick ✓ / △ / ✗ / N/A for each row
-• Score auto-totals at the bottom
-• Log the chart on the Audit Log tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+1. Fill in the yellow cells at top
+2. Rate each element (dropdown in column C)
+3. Overall % + Rating appear at the bottom
+4. Log the chart on the Audit Log tab when done</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>MRN (masked):</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Category:</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Payer:</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="7" ht="12" customHeight="1"/>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>§</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Documentation Element</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Documentation element</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>Notes / evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A · Diagnosis Accuracy   (4 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>All reported diagnoses are clinically supported in the note</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="9">
-        <f>IF(C9="✓ Met",1,IF(C9="△ Partial",0.5,IF(C9="✗ Not Met",0,IF(C9="N/A","",""))))</f>
-        <v/>
-      </c>
-      <c r="E9" s="10" t="n"/>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Chronic conditions actively addressed at this visit (not just carried forward)</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="9">
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33">
         <f>IF(C10="✓ Met",1,IF(C10="△ Partial",0.5,IF(C10="✗ Not Met",0,IF(C10="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E10" s="10" t="n"/>
     </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>A3</t>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>A2</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>No unsupported or resolved conditions billed as active</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="9">
+          <t>Chronic conditions actively addressed at this visit (not just carried forward)</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="33">
         <f>IF(C11="✓ Met",1,IF(C11="△ Partial",0.5,IF(C11="✗ Not Met",0,IF(C11="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E11" s="10" t="n"/>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>A4</t>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>A3</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Problem list matches today's assessment &amp; plan</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="9">
+          <t>No unsupported or resolved conditions billed as active</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="33">
         <f>IF(C12="✓ Met",1,IF(C12="△ Partial",0.5,IF(C12="✗ Not Met",0,IF(C12="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E12" s="10" t="n"/>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>ICD-10 codes at highest available specificity (avoid 'unspecified')</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="9">
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Problem list matches today's assessment &amp; plan</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="33">
         <f>IF(C13="✓ Met",1,IF(C13="△ Partial",0.5,IF(C13="✗ Not Met",0,IF(C13="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E13" s="10" t="n"/>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Diabetes: type + complications + control specified</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="9">
-        <f>IF(C14="✓ Met",1,IF(C14="△ Partial",0.5,IF(C14="✗ Not Met",0,IF(C14="N/A","",""))))</f>
-        <v/>
-      </c>
-      <c r="E14" s="10" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>S / O / A / P sections tell one consistent clinical story</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="9">
-        <f>IF(C15="✓ Met",1,IF(C15="△ Partial",0.5,IF(C15="✗ Not Met",0,IF(C15="N/A","",""))))</f>
-        <v/>
-      </c>
-      <c r="E15" s="10" t="n"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>B4</t>
+    <row r="14" ht="6" customHeight="1"/>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B · Documentation Specificity   (4 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>B1</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Note signed, dated, and closed by the rendering provider</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="9">
+          <t>ICD-10 codes at highest available specificity (avoid 'unspecified')</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="33">
         <f>IF(C16="✓ Met",1,IF(C16="△ Partial",0.5,IF(C16="✗ Not Met",0,IF(C16="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E16" s="10" t="n"/>
     </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Monitor — signs, symptoms, or labs monitored</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="9">
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Diabetes: type + complications + control specified</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="33">
         <f>IF(C17="✓ Met",1,IF(C17="△ Partial",0.5,IF(C17="✗ Not Met",0,IF(C17="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E17" s="10" t="n"/>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>C2</t>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>B3</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Evaluate — response to treatment evaluated</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="9">
+          <t>S / O / A / P sections tell one consistent clinical story</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="33">
         <f>IF(C18="✓ Met",1,IF(C18="△ Partial",0.5,IF(C18="✗ Not Met",0,IF(C18="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E18" s="10" t="n"/>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>C3</t>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>B4</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Assess / Address — diagnosis explicitly assessed today</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="9">
+          <t>Note signed, dated, and closed by the rendering provider</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="33">
         <f>IF(C19="✓ Met",1,IF(C19="△ Partial",0.5,IF(C19="✗ Not Met",0,IF(C19="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E19" s="10" t="n"/>
     </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Treat — treatment plan documented (med / referral / testing / follow-up)</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9">
-        <f>IF(C20="✓ Met",1,IF(C20="△ Partial",0.5,IF(C20="✗ Not Met",0,IF(C20="N/A","",""))))</f>
-        <v/>
-      </c>
-      <c r="E20" s="10" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Prior-year HCCs recaptured (or explicitly resolved with rationale)</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9">
-        <f>IF(C21="✓ Met",1,IF(C21="△ Partial",0.5,IF(C21="✗ Not Met",0,IF(C21="N/A","",""))))</f>
-        <v/>
-      </c>
-      <c r="E21" s="10" t="n"/>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>D2</t>
+    <row r="20" ht="6" customHeight="1"/>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C · MEAT Support   (4 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>C1</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Suspected undocumented chronic conditions captured with support</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9">
+          <t>Monitor — signs, symptoms, or labs monitored</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="33">
         <f>IF(C22="✓ Met",1,IF(C22="△ Partial",0.5,IF(C22="✗ Not Met",0,IF(C22="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E22" s="10" t="n"/>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Applicable CPT II codes reported for open quality measures</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9">
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Evaluate — response to treatment evaluated</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="33">
         <f>IF(C23="✓ Met",1,IF(C23="△ Partial",0.5,IF(C23="✗ Not Met",0,IF(C23="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E23" s="10" t="n"/>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>E2</t>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>C3</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Reason modifiers (1P / 2P / 3P / 8P) applied when measure not met</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9">
+          <t>Assess / Address — diagnosis explicitly assessed today</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="33">
         <f>IF(C24="✓ Met",1,IF(C24="△ Partial",0.5,IF(C24="✗ Not Met",0,IF(C24="N/A","",""))))</f>
         <v/>
       </c>
       <c r="E24" s="10" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Treat — treatment plan documented (medication / referral / testing / follow-up)</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="33">
+        <f>IF(C25="✓ Met",1,IF(C25="△ Partial",0.5,IF(C25="✗ Not Met",0,IF(C25="N/A","",""))))</f>
+        <v/>
+      </c>
+      <c r="E25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="6" customHeight="1"/>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D · HCC Capture   (2 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Prior-year HCCs recaptured (or explicitly resolved with rationale)</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="33">
+        <f>IF(C28="✓ Met",1,IF(C28="△ Partial",0.5,IF(C28="✗ Not Met",0,IF(C28="N/A","",""))))</f>
+        <v/>
+      </c>
+      <c r="E28" s="10" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Suspected undocumented chronic conditions captured with support</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="33">
+        <f>IF(C29="✓ Met",1,IF(C29="△ Partial",0.5,IF(C29="✗ Not Met",0,IF(C29="N/A","",""))))</f>
+        <v/>
+      </c>
+      <c r="E29" s="10" t="n"/>
+    </row>
+    <row r="30" ht="6" customHeight="1"/>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E · CPT II Reporting   (2 items)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Applicable CPT II codes reported for open quality measures</t>
+        </is>
+      </c>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="33">
+        <f>IF(C32="✓ Met",1,IF(C32="△ Partial",0.5,IF(C32="✗ Not Met",0,IF(C32="N/A","",""))))</f>
+        <v/>
+      </c>
+      <c r="E32" s="10" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Reason modifiers (1P / 2P / 3P / 8P) applied when a measure is not met</t>
+        </is>
+      </c>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="33">
+        <f>IF(C33="✓ Met",1,IF(C33="△ Partial",0.5,IF(C33="✗ Not Met",0,IF(C33="N/A","",""))))</f>
+        <v/>
+      </c>
+      <c r="E33" s="10" t="n"/>
+    </row>
+    <row r="34" ht="6" customHeight="1"/>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>§</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Applicable</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>% Met</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="35" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B28" s="11" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Diagnosis Accuracy</t>
         </is>
       </c>
-      <c r="C28" s="9">
-        <f>COUNTIF(C9:C12,"✓ Met")+COUNTIF(C9:C12,"△ Partial")+COUNTIF(C9:C12,"✗ Not Met")</f>
+      <c r="C38" s="36">
+        <f>COUNTIF(C10:C13,"✓ Met")+COUNTIF(C10:C13,"△ Partial")+COUNTIF(C10:C13,"✗ Not Met")</f>
         <v/>
       </c>
-      <c r="D28" s="12">
-        <f>IFERROR(SUM(D9:D12)/C28,"")</f>
+      <c r="D38" s="37">
+        <f>IFERROR(SUM(D10:D13)/C38,"")</f>
         <v/>
       </c>
-      <c r="E28" s="10" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr"/>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="35" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Documentation Specificity</t>
         </is>
       </c>
-      <c r="C29" s="9">
-        <f>COUNTIF(C13:C16,"✓ Met")+COUNTIF(C13:C16,"△ Partial")+COUNTIF(C13:C16,"✗ Not Met")</f>
+      <c r="C39" s="36">
+        <f>COUNTIF(C16:C19,"✓ Met")+COUNTIF(C16:C19,"△ Partial")+COUNTIF(C16:C19,"✗ Not Met")</f>
         <v/>
       </c>
-      <c r="D29" s="12">
-        <f>IFERROR(SUM(D13:D16)/C29,"")</f>
+      <c r="D39" s="37">
+        <f>IFERROR(SUM(D16:D19)/C39,"")</f>
         <v/>
       </c>
-      <c r="E29" s="10" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr"/>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="35" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>MEAT Support</t>
         </is>
       </c>
-      <c r="C30" s="9">
-        <f>COUNTIF(C17:C20,"✓ Met")+COUNTIF(C17:C20,"△ Partial")+COUNTIF(C17:C20,"✗ Not Met")</f>
+      <c r="C40" s="36">
+        <f>COUNTIF(C22:C25,"✓ Met")+COUNTIF(C22:C25,"△ Partial")+COUNTIF(C22:C25,"✗ Not Met")</f>
         <v/>
       </c>
-      <c r="D30" s="12">
-        <f>IFERROR(SUM(D17:D20)/C30,"")</f>
+      <c r="D40" s="37">
+        <f>IFERROR(SUM(D22:D25)/C40,"")</f>
         <v/>
       </c>
-      <c r="E30" s="10" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="E40" s="14" t="inlineStr"/>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="35" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>HCC Capture</t>
         </is>
       </c>
-      <c r="C31" s="9">
-        <f>COUNTIF(C21:C22,"✓ Met")+COUNTIF(C21:C22,"△ Partial")+COUNTIF(C21:C22,"✗ Not Met")</f>
+      <c r="C41" s="36">
+        <f>COUNTIF(C28:C29,"✓ Met")+COUNTIF(C28:C29,"△ Partial")+COUNTIF(C28:C29,"✗ Not Met")</f>
         <v/>
       </c>
-      <c r="D31" s="12">
-        <f>IFERROR(SUM(D21:D22)/C31,"")</f>
+      <c r="D41" s="37">
+        <f>IFERROR(SUM(D28:D29)/C41,"")</f>
         <v/>
       </c>
-      <c r="E31" s="10" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr"/>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="35" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>CPT II Reporting</t>
         </is>
       </c>
-      <c r="C32" s="9">
-        <f>COUNTIF(C23:C24,"✓ Met")+COUNTIF(C23:C24,"△ Partial")+COUNTIF(C23:C24,"✗ Not Met")</f>
+      <c r="C42" s="36">
+        <f>COUNTIF(C32:C33,"✓ Met")+COUNTIF(C32:C33,"△ Partial")+COUNTIF(C32:C33,"✗ Not Met")</f>
         <v/>
       </c>
-      <c r="D32" s="12">
-        <f>IFERROR(SUM(D23:D24)/C32,"")</f>
+      <c r="D42" s="37">
+        <f>IFERROR(SUM(D32:D33)/C42,"")</f>
         <v/>
       </c>
-      <c r="E32" s="10" t="n"/>
-    </row>
-    <row r="34" ht="34" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>OVERALL COMPLIANCE %</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="15">
-        <f>SUM(C28:C32)</f>
+      <c r="E42" s="14" t="inlineStr"/>
+    </row>
+    <row r="44" ht="44" customHeight="1">
+      <c r="A44" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OVERALL COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="D44" s="39">
+        <f>IFERROR(SUMPRODUCT(D38:D42,C38:C42)/SUM(C38:C42),"")</f>
         <v/>
       </c>
-      <c r="D34" s="16">
-        <f>IFERROR(SUMPRODUCT(D28:D32,C28:C32)/SUM(C28:C32),"")</f>
+      <c r="E44" s="17" t="n"/>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PERFORMANCE BAND</t>
+        </is>
+      </c>
+      <c r="D45" s="18">
+        <f>IF(D44="","",IF(D44&gt;=0.95,"Excellent",IF(D44&gt;=0.90,"Meets Expectations",IF(D44&gt;=0.80,"Needs Improvement","Corrective Education Required"))))</f>
         <v/>
       </c>
-      <c r="E34" s="17" t="n"/>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>RATING</t>
-        </is>
-      </c>
-      <c r="D35" s="18">
-        <f>IF(D34="","",IF(D34&gt;=0.95,"Excellent",IF(D34&gt;=0.90,"Meets Expectations",IF(D34&gt;=0.80,"Needs Improvement","Corrective Education Required"))))</f>
-        <v/>
-      </c>
-      <c r="E35" s="14" t="n"/>
+      <c r="E45" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="11">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="E4:E6"/>
-    <mergeCell ref="E6"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
-  <conditionalFormatting sqref="C9:C24">
+  <conditionalFormatting sqref="C10:C34">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>C9="✓ Met"</formula>
+      <formula>C10="✓ Met"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>C9="△ Partial"</formula>
+      <formula>C10="△ Partial"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>C9="✗ Not Met"</formula>
+      <formula>C10="✗ Not Met"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>C9="N/A"</formula>
+      <formula>C10="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D28">
+  <conditionalFormatting sqref="D38">
     <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
@@ -1215,7 +1443,7 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D29">
+  <conditionalFormatting sqref="D39">
     <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
@@ -1227,7 +1455,7 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D30">
+  <conditionalFormatting sqref="D40">
     <cfRule type="cellIs" priority="11" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
@@ -1239,7 +1467,7 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D31">
+  <conditionalFormatting sqref="D41">
     <cfRule type="cellIs" priority="14" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
@@ -1251,7 +1479,7 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D32">
+  <conditionalFormatting sqref="D42">
     <cfRule type="cellIs" priority="17" operator="greaterThanOrEqual" dxfId="0">
       <formula>0.9</formula>
     </cfRule>
@@ -1263,7 +1491,7 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D34">
+  <conditionalFormatting sqref="D44">
     <cfRule type="cellIs" priority="20" operator="greaterThanOrEqual" dxfId="3">
       <formula>0.95</formula>
     </cfRule>
@@ -1279,18 +1507,18 @@
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35">
+  <conditionalFormatting sqref="D45">
     <cfRule type="expression" priority="24" dxfId="3">
-      <formula>D35="Excellent"</formula>
+      <formula>D45="Excellent"</formula>
     </cfRule>
     <cfRule type="expression" priority="25" dxfId="0">
-      <formula>D35="Meets Expectations"</formula>
+      <formula>D45="Meets Expectations"</formula>
     </cfRule>
     <cfRule type="expression" priority="26" dxfId="1">
-      <formula>D35="Needs Improvement"</formula>
+      <formula>D45="Needs Improvement"</formula>
     </cfRule>
     <cfRule type="expression" priority="27" dxfId="2">
-      <formula>D35="Corrective Education Required"</formula>
+      <formula>D45="Corrective Education Required"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -1300,7 +1528,7 @@
     <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
     </dataValidation>
-    <dataValidation sqref="C9:C24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Replace section C MEAT with SOAP note structure
Audit Checklist section C is now SOAP (Subjective / Objective /
Assessment / Plan) instead of MEAT. Quick Reference SOAP block
updated with matching examples.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -1079,7 +1079,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  C · MEAT Support   (4 items)</t>
+          <t xml:space="preserve">  C · SOAP Note Structure   (4 items)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Monitor — signs, symptoms, or labs monitored</t>
+          <t>Subjective — patient's history, symptoms, and concerns clearly documented</t>
         </is>
       </c>
       <c r="C22" s="32" t="n"/>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Evaluate — response to treatment evaluated</t>
+          <t>Objective — exam findings, vitals, and relevant test results documented</t>
         </is>
       </c>
       <c r="C23" s="32" t="n"/>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Assess / Address — diagnosis explicitly assessed today</t>
+          <t>Assessment — each diagnosis explicitly assessed with clinical reasoning</t>
         </is>
       </c>
       <c r="C24" s="32" t="n"/>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Treat — treatment plan documented (medication / referral / testing / follow-up)</t>
+          <t>Plan — treatment plan documented (medication / referral / testing / follow-up)</t>
         </is>
       </c>
       <c r="C25" s="32" t="n"/>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>MEAT Support</t>
+          <t>SOAP Note Structure</t>
         </is>
       </c>
       <c r="C40" s="36">
@@ -3842,14 +3842,14 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Quick Reference — MEAT · Bands · High-Risk Dx · CPT II</t>
+          <t>Quick Reference — SOAP · Bands · High-Risk Dx · CPT II</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>MEAT Criteria</t>
+          <t>SOAP Note Structure</t>
         </is>
       </c>
     </row>
@@ -3874,17 +3874,17 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Monitor</t>
+          <t>Subjective</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Signs / symptoms / labs monitored</t>
+          <t>Patient history, symptoms, concerns</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HbA1c 7.8 stable, BP log reviewed</t>
+          <t>'Patient reports 2-week low mood, poor sleep, denies SI/HI'</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr"/>
@@ -3892,17 +3892,17 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Evaluate</t>
+          <t>Objective</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Response to treatment evaluated</t>
+          <t>Exam findings, vitals, labs, screening scores</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>BP controlled on lisinopril</t>
+          <t>'BP 128/82, PHQ-9 = 14, GAD-7 = 9, MSE alert &amp; oriented'</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr"/>
@@ -3910,17 +3910,17 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Assess / Address</t>
+          <t>Assessment</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Diagnosis reviewed and addressed</t>
+          <t>Diagnosis with clinical reasoning</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>DM Type 2 with neuropathy — ongoing</t>
+          <t>'MDD moderate (F32.1) — partial response; GAD (F41.1) stable'</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr"/>
@@ -3928,17 +3928,17 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Treat</t>
+          <t>Plan</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Treatment plan documented</t>
+          <t>Treatment plan documented in full</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Continue metformin 1000 mg BID; recheck A1c 3 mo</t>
+          <t>'Continue escitalopram 10 mg; CBT weekly; recheck PHQ-9 in 4 wk'</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Rename MRN to Claim Number and add Quarterly Report tab
- Row 5 label on Audit Checklist and column C on Audit Log now say
  'Claim Number' instead of 'MRN (masked)'.
- New Quarterly Report tab: quarter + year picker, 4 KPI tiles
  (charts audited, avg compliance %, meeting expectations, corrective
  required), and 4 charts (band bar chart, category pie, monthly
  compliance line, charts-per-month bar) driven by SUMPRODUCT queries
  against the Audit Log.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Audit Checklist" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Audit Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Quick Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Quarterly Report" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +132,32 @@
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="22"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -187,6 +212,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000B5555"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F7FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -298,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -416,6 +446,28 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,6 +572,447 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="11"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charts by Performance Band</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!C11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$B$12:$B$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$C$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charts by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!F11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$E$12:$E$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$F$12:$F$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly Compliance % Trend</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!J11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$H$12:$H$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$J$12:$J$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Avg Compliance %</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Charts Audited per Month</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!I11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$H$12:$H$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$I$12:$I$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -863,7 +1356,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>MRN (masked):</t>
+          <t>Claim Number:</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
@@ -1586,7 +2079,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>MRN (masked)</t>
+          <t>Claim Number</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -4570,4 +5063,340 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00B45309"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Quarterly Audit Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Pick a quarter &amp; year — metrics and charts recalculate from the Audit Log automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Quarter:</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Year:</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H4" s="42" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="I4" s="9">
+        <f>CHOOSE(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0),"Jan – Mar","Apr – Jun","Jul – Sep","Oct – Dec")</f>
+        <v/>
+      </c>
+      <c r="J4" s="43">
+        <f>$E$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>Charts Audited</t>
+        </is>
+      </c>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="44" t="inlineStr">
+        <is>
+          <t>Avg Compliance %</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="n"/>
+      <c r="F6" s="44" t="inlineStr">
+        <is>
+          <t>Meeting Expectations (≥90%)</t>
+        </is>
+      </c>
+      <c r="G6" s="45" t="n"/>
+      <c r="H6" s="44" t="inlineStr">
+        <is>
+          <t>Corrective Required (&lt;80%)</t>
+        </is>
+      </c>
+      <c r="I6" s="45" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="46">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*1)</f>
+        <v/>
+      </c>
+      <c r="D7" s="47">
+        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="46">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&gt;=0.9))</f>
+        <v/>
+      </c>
+      <c r="H7" s="46">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;0.8)*('Audit Log'!$F$5:$F$200&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="14" t="n"/>
+    </row>
+    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="26" customHeight="1">
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>Charts by Performance Band</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="n"/>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>Charts by Category</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="n"/>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>Monthly Trend — Avg Compliance %</t>
+        </is>
+      </c>
+      <c r="I10" s="45" t="n"/>
+      <c r="J10" s="45" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Charts</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Avg %</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="C12" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Excellent"))</f>
+        <v/>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="F12" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Diabetes"))</f>
+        <v/>
+      </c>
+      <c r="H12" s="9">
+        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1,1),"mmm yyyy")</f>
+        <v/>
+      </c>
+      <c r="I12" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
+        <v/>
+      </c>
+      <c r="J12" s="37">
+        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="C13" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Meets Expectations"))</f>
+        <v/>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Chronic Kidney Disease</t>
+        </is>
+      </c>
+      <c r="F13" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Chronic Kidney Disease"))</f>
+        <v/>
+      </c>
+      <c r="H13" s="9">
+        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2,1),"mmm yyyy")</f>
+        <v/>
+      </c>
+      <c r="I13" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
+        <v/>
+      </c>
+      <c r="J13" s="37">
+        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+      <c r="C14" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Needs Improvement"))</f>
+        <v/>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Annual Wellness Visit</t>
+        </is>
+      </c>
+      <c r="F14" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Annual Wellness Visit"))</f>
+        <v/>
+      </c>
+      <c r="H14" s="9">
+        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3,1),"mmm yyyy")</f>
+        <v/>
+      </c>
+      <c r="I14" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
+        <v/>
+      </c>
+      <c r="J14" s="37">
+        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Corrective Education Required</t>
+        </is>
+      </c>
+      <c r="C15" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Corrective Education Required"))</f>
+        <v/>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>High RAF Patient</t>
+        </is>
+      </c>
+      <c r="F15" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="High RAF Patient"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Random Selection</t>
+        </is>
+      </c>
+      <c r="F16" s="33">
+        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Random Selection"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="D7:E8"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="F7:G8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Q1,Q2,Q3,Q4"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Reframe section E — audit documentation, not billing codes
Section E now titled 'Documentation Supporting Quality Measures'.
Audits whether the provider's note gives the billing team what they
need for CPT II capture, rather than whether the code was reported.

E1 — Screening/measure results documented with specific values
     (PHQ-9, GAD-7, BMI, BP, HbA1c) rather than 'screened'/'normal'.
E2 — Follow-up plan documented when a result is positive/abnormal.

Quick Reference CPT II block gets a matching header note clarifying
that the billing team assigns the codes and the auditor's job is to
verify the documentation supports that assignment.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -156,6 +156,12 @@
       <color rgb="000F172A"/>
       <sz val="22"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -220,7 +226,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -324,11 +330,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -466,6 +503,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1696,7 +1739,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  E · CPT II Reporting   (2 items)</t>
+          <t xml:space="preserve">  E · Documentation Supporting Quality Measures   (2 items)</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1751,7 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Applicable CPT II codes reported for open quality measures</t>
+          <t>Screening / measure results documented with specific values (PHQ-9, GAD-7, BMI, BP, HbA1c) — not just 'screened' or 'normal'</t>
         </is>
       </c>
       <c r="C32" s="32" t="n"/>
@@ -1726,7 +1769,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Reason modifiers (1P / 2P / 3P / 8P) applied when a measure is not met</t>
+          <t>Follow-up plan documented when a screening is positive or a result is abnormal (positive PHQ-9 → depression plan; elevated BMI → nutrition counseling)</t>
         </is>
       </c>
       <c r="C33" s="32" t="n"/>
@@ -1859,7 +1902,7 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>CPT II Reporting</t>
+          <t>Documentation Supporting Quality Measures</t>
         </is>
       </c>
       <c r="C42" s="36">
@@ -4323,7 +4366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4805,131 +4848,95 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="20" t="inlineStr">
-        <is>
-          <t>CPT II Priority Measures</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Documentation Needed for CPT II Capture</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>The billing team assigns the codes below — your job is to document the specific value AND the follow-up action so they can capture the measure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="6" customHeight="1"/>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>CPT II Codes</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>HbA1c control (DM)</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>3044F / 3046F / 3051F / 3052F</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>Diabetes patients</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>Report per most recent A1c</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>BP control (HTN)</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>3074F / 3075F / 3077F / 3078F</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>Hypertension patients</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>Document sys &amp; dias</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>BMI screening + follow-up</t>
+          <t>HbA1c control (DM)</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>G8417 / G8418 / G8420</t>
+          <t>3044F / 3046F / 3051F / 3052F</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>All adult visits</t>
+          <t>Diabetes patients</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Include intervention if abnormal</t>
+          <t>Report per most recent A1c</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Tobacco screening + cessation</t>
+          <t>BP control (HTN)</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>1036F / 4004F</t>
+          <t>3074F / 3075F / 3077F / 3078F</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>All adult visits</t>
+          <t>Hypertension patients</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Screening + counseling combo</t>
+          <t>Document sys &amp; dias</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Depression screening + plan</t>
+          <t>BMI screening + follow-up</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>G8431 / G8510</t>
+          <t>G8417 / G8418 / G8420</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -4939,127 +4946,172 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>PHQ-2 / PHQ-9 documented</t>
+          <t>Include intervention if abnormal</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Statin therapy for CVD</t>
+          <t>Tobacco screening + cessation</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>0521F / 4013F</t>
+          <t>1036F / 4004F</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>ASCVD / DM / LDL ≥190</t>
+          <t>All adult visits</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>On statin, refused, or contraindicated</t>
+          <t>Screening + counseling combo</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>Diabetic eye exam</t>
+          <t>Depression screening + plan</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>2022F / 2024F / 2026F</t>
+          <t>G8431 / G8510</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Diabetes patients</t>
+          <t>All adult visits</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Negative or positive result</t>
+          <t>PHQ-2 / PHQ-9 documented</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Nephropathy screening</t>
+          <t>Statin therapy for CVD</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>3060F / 3061F / 3062F</t>
+          <t>0521F / 4013F</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Diabetes patients</t>
+          <t>ASCVD / DM / LDL ≥190</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Urine albumin / on ACE-ARB</t>
+          <t>On statin, refused, or contraindicated</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Med rec post-discharge</t>
+          <t>Diabetic eye exam</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>1111F</t>
+          <t>2022F / 2024F / 2026F</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Discharge in last 30 d</t>
+          <t>Diabetes patients</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Reconciliation documented</t>
+          <t>Negative or positive result</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
+          <t>Nephropathy screening</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>3060F / 3061F / 3062F</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Diabetes patients</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Urine albumin / on ACE-ARB</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>Med rec post-discharge</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>1111F</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Discharge in last 30 d</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Reconciliation documented</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
           <t>Fall risk assessment</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>1101F</t>
         </is>
       </c>
-      <c r="C42" s="10" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Age 65+</t>
         </is>
       </c>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>Yearly for MA populations</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Quarterly Report charts + seed Audit Log with sample data
- Rebuild all 4 charts with non-overlapping anchors (B18 / H18 / B36 /
  H36), larger sizes, integer y-axis format on count charts, and a
  fixed 60-100% y-axis on the compliance-trend line so movement is
  visible even in a narrow range.
- Add circle markers to the line chart.
- Seed the Audit Log with 10 realistic sample rows (highlighted so the
  auditor can spot and delete them before entering real audits) — this
  gives the Quarterly Report visible data on first open.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -163,7 +164,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -223,6 +224,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -365,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -511,6 +517,25 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -704,9 +729,11 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="1"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -761,6 +788,7 @@
           </val>
         </ser>
         <dLbls>
+          <showCatName val="0"/>
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>
@@ -810,7 +838,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="8"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -849,6 +878,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="1"/>
+          <min val="0.6"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
@@ -873,9 +904,6 @@
         <crossAx val="10"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -954,9 +982,11 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="1"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -974,7 +1004,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3240000"/>
+    <ext cx="5400000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -991,12 +1021,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1015,10 +1045,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3240000"/>
+    <ext cx="5400000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1035,12 +1065,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>36</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1409,6 +1439,7 @@
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
+      <c r="E5" s="51" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
@@ -1423,6 +1454,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
+      <c r="E6" s="52" t="n"/>
     </row>
     <row r="7" ht="12" customHeight="1"/>
     <row r="8" ht="32" customHeight="1">
@@ -1933,6 +1965,8 @@
           <t xml:space="preserve">  PERFORMANCE BAND</t>
         </is>
       </c>
+      <c r="B45" s="53" t="n"/>
+      <c r="C45" s="54" t="n"/>
       <c r="D45" s="18">
         <f>IF(D44="","",IF(D44&gt;=0.95,"Excellent",IF(D44&gt;=0.90,"Meets Expectations",IF(D44&gt;=0.80,"Needs Improvement","Corrective Education Required"))))</f>
         <v/>
@@ -2157,114 +2191,414 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="9" t="n"/>
-      <c r="F5" s="12" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
+      <c r="A5" s="55" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-001</t>
+        </is>
+      </c>
+      <c r="D5" s="55" t="n">
+        <v>46201</v>
+      </c>
+      <c r="E5" s="57" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="F5" s="58" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G5" s="57" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="H5" s="56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I5" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="12" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
+      <c r="A6" s="55" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C6" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-002</t>
+        </is>
+      </c>
+      <c r="D6" s="55" t="n">
+        <v>46203</v>
+      </c>
+      <c r="E6" s="57" t="inlineStr">
+        <is>
+          <t>Chronic Kidney Disease</t>
+        </is>
+      </c>
+      <c r="F6" s="58" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G6" s="57" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="H6" s="56" t="inlineStr">
+        <is>
+          <t>N18 unspecified</t>
+        </is>
+      </c>
+      <c r="I6" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n"/>
+      <c r="A7" s="55" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C7" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-003</t>
+        </is>
+      </c>
+      <c r="D7" s="55" t="n">
+        <v>46208</v>
+      </c>
+      <c r="E7" s="57" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G7" s="57" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+      <c r="H7" s="56" t="inlineStr">
+        <is>
+          <t>E11.9 use, missing MEAT</t>
+        </is>
+      </c>
+      <c r="I7" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
+      <c r="A8" s="55" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C8" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-004</t>
+        </is>
+      </c>
+      <c r="D8" s="55" t="n">
+        <v>46212</v>
+      </c>
+      <c r="E8" s="57" t="inlineStr">
+        <is>
+          <t>Annual Wellness Visit</t>
+        </is>
+      </c>
+      <c r="F8" s="58" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G8" s="57" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="H8" s="56" t="inlineStr">
+        <is>
+          <t>PHQ-9 score not documented</t>
+        </is>
+      </c>
+      <c r="I8" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
+      <c r="A9" s="55" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-005</t>
+        </is>
+      </c>
+      <c r="D9" s="55" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E9" s="57" t="inlineStr">
+        <is>
+          <t>High RAF Patient</t>
+        </is>
+      </c>
+      <c r="F9" s="58" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G9" s="57" t="inlineStr">
+        <is>
+          <t>Corrective Education Required</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="inlineStr">
+        <is>
+          <t>HCC recapture missed</t>
+        </is>
+      </c>
+      <c r="I9" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
+      <c r="A10" s="55" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C10" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-006</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="n">
+        <v>46238</v>
+      </c>
+      <c r="E10" s="57" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="F10" s="58" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G10" s="57" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="H10" s="56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I10" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
+      <c r="A11" s="55" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C11" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-007</t>
+        </is>
+      </c>
+      <c r="D11" s="55" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E11" s="57" t="inlineStr">
+        <is>
+          <t>Chronic Kidney Disease</t>
+        </is>
+      </c>
+      <c r="F11" s="58" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G11" s="57" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="inlineStr">
+        <is>
+          <t>CKD stage unspecified</t>
+        </is>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n"/>
+      <c r="A12" s="55" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B12" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C12" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-008</t>
+        </is>
+      </c>
+      <c r="D12" s="55" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E12" s="57" t="inlineStr">
+        <is>
+          <t>Annual Wellness Visit</t>
+        </is>
+      </c>
+      <c r="F12" s="58" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G12" s="57" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="H12" s="56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I12" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="10" t="n"/>
+      <c r="A13" s="55" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-009</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E13" s="57" t="inlineStr">
+        <is>
+          <t>Random Selection</t>
+        </is>
+      </c>
+      <c r="F13" s="58" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G13" s="57" t="inlineStr">
+        <is>
+          <t>Needs Improvement</t>
+        </is>
+      </c>
+      <c r="H13" s="56" t="inlineStr">
+        <is>
+          <t>Med rec not documented</t>
+        </is>
+      </c>
+      <c r="I13" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n"/>
+      <c r="A14" s="55" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C14" s="56" t="inlineStr">
+        <is>
+          <t>CLM-2026-010</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E14" s="57" t="inlineStr">
+        <is>
+          <t>High RAF Patient</t>
+        </is>
+      </c>
+      <c r="F14" s="58" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G14" s="57" t="inlineStr">
+        <is>
+          <t>Meets Expectations</t>
+        </is>
+      </c>
+      <c r="H14" s="56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I14" s="56" t="inlineStr">
+        <is>
+          <t>Sample row · delete when starting real audits</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n"/>
@@ -4860,6 +5194,9 @@
           <t>The billing team assigns the codes below — your job is to document the specific value AND the follow-up action so they can capture the measure.</t>
         </is>
       </c>
+      <c r="B32" s="53" t="n"/>
+      <c r="C32" s="53" t="n"/>
+      <c r="D32" s="54" t="n"/>
     </row>
     <row r="33" ht="6" customHeight="1"/>
     <row r="34">
@@ -5129,10 +5466,10 @@
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="4" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -5193,53 +5530,57 @@
           <t>Charts Audited</t>
         </is>
       </c>
-      <c r="C6" s="45" t="n"/>
+      <c r="C6" s="54" t="n"/>
       <c r="D6" s="44" t="inlineStr">
         <is>
           <t>Avg Compliance %</t>
         </is>
       </c>
-      <c r="E6" s="45" t="n"/>
+      <c r="E6" s="54" t="n"/>
       <c r="F6" s="44" t="inlineStr">
         <is>
           <t>Meeting Expectations (≥90%)</t>
         </is>
       </c>
-      <c r="G6" s="45" t="n"/>
+      <c r="G6" s="54" t="n"/>
       <c r="H6" s="44" t="inlineStr">
         <is>
           <t>Corrective Required (&lt;80%)</t>
         </is>
       </c>
-      <c r="I6" s="45" t="n"/>
+      <c r="I6" s="54" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="B7" s="46">
         <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*1)</f>
         <v/>
       </c>
+      <c r="C7" s="59" t="n"/>
       <c r="D7" s="47">
         <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),"")</f>
         <v/>
       </c>
+      <c r="E7" s="59" t="n"/>
       <c r="F7" s="46">
         <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&gt;=0.9))</f>
         <v/>
       </c>
+      <c r="G7" s="59" t="n"/>
       <c r="H7" s="46">
         <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;0.8)*('Audit Log'!$F$5:$F$200&lt;&gt;""))</f>
         <v/>
       </c>
+      <c r="I7" s="59" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="n"/>
+      <c r="B8" s="60" t="n"/>
+      <c r="C8" s="61" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="61" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="61" t="n"/>
+      <c r="H8" s="60" t="n"/>
+      <c r="I8" s="61" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="26" customHeight="1">
@@ -5248,20 +5589,20 @@
           <t>Charts by Performance Band</t>
         </is>
       </c>
-      <c r="C10" s="45" t="n"/>
+      <c r="C10" s="54" t="n"/>
       <c r="E10" s="48" t="inlineStr">
         <is>
           <t>Charts by Category</t>
         </is>
       </c>
-      <c r="F10" s="45" t="n"/>
+      <c r="F10" s="54" t="n"/>
       <c r="H10" s="48" t="inlineStr">
         <is>
           <t>Monthly Trend — Avg Compliance %</t>
         </is>
       </c>
-      <c r="I10" s="45" t="n"/>
-      <c r="J10" s="45" t="n"/>
+      <c r="I10" s="53" t="n"/>
+      <c r="J10" s="54" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="7" t="inlineStr">
@@ -5427,6 +5768,43 @@
         <v/>
       </c>
     </row>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="18" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1"/>
+    <row r="27" ht="18" customHeight="1"/>
+    <row r="28" ht="18" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="18" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1"/>
+    <row r="32" ht="18" customHeight="1"/>
+    <row r="33" ht="18" customHeight="1"/>
+    <row r="34" ht="18" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1"/>
+    <row r="36" ht="18" customHeight="1"/>
+    <row r="37" ht="18" customHeight="1"/>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1"/>
+    <row r="48" ht="18" customHeight="1"/>
+    <row r="49" ht="18" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="18" customHeight="1"/>
+    <row r="53" ht="18" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="D6:E6"/>

</xml_diff>

<commit_message>
Simplify Quarterly Report to a single provider-progression view
Replaced the 4 old charts (band bar, category pie, monthly trend line,
monthly volume bar) and their supporting data tables with:
- A Provider Progression table: 5 provider slots × 12 months of the
  selected year, showing each provider's monthly average compliance %,
  color-coded (green >=90, amber 80-89, red <80).
- A single line chart with one line per provider so you can see who
  is improving and who is declining across the year at a glance.

KPI tiles at the top (charts audited, avg compliance %, meeting
expectations, corrective required) are unchanged.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -161,6 +161,13 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font/>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000B5555"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -371,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -536,6 +543,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -644,7 +667,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="11"/>
   <chart>
     <title>
       <tx>
@@ -655,167 +677,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Charts by Performance Band</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Quarterly Report'!C11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Quarterly Report'!$B$12:$B$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Quarterly Report'!$C$12:$C$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Count</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <majorUnit val="1"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Charts by Category</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Quarterly Report'!F11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Quarterly Report'!$E$12:$E$16</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Quarterly Report'!$F$12:$F$16</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showCatName val="0"/>
-          <showPercent val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Monthly Compliance % Trend</a:t>
+              <a:t>Provider Compliance % Progression</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -829,7 +691,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Quarterly Report'!J11</f>
+              <f>'Quarterly Report'!B12</f>
             </strRef>
           </tx>
           <spPr>
@@ -839,7 +701,7 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
-            <size val="8"/>
+            <size val="7"/>
             <spPr>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -848,17 +710,182 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Quarterly Report'!$H$12:$H$14</f>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Quarterly Report'!$J$12:$J$14</f>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!B13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$13:$N$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!B14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$14:$N$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!B15</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$15:$N$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!B16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$16:$N$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Quarterly Report'!B17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Quarterly Report'!$C$12:$N$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Quarterly Report'!$C$17:$N$17</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
-          <showVal val="1"/>
+          <showVal val="0"/>
         </dLbls>
         <axId val="10"/>
         <axId val="100"/>
@@ -892,7 +919,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Avg Compliance %</a:t>
+                  <a:t>Compliance %</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -902,93 +929,12 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="0.05"/>
       </valAx>
     </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Charts Audited per Month</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Quarterly Report'!I11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Quarterly Report'!$H$12:$H$14</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Quarterly Report'!$I$12:$I$14</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <majorUnit val="1"/>
-      </valAx>
-    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -1001,10 +947,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>17</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="3060000"/>
+    <ext cx="10080000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1014,72 +960,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="3060000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="3060000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>35</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="3060000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="4" name="Chart 4"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -5461,19 +5341,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="4" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="3" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -5582,189 +5467,375 @@
       <c r="H8" s="60" t="n"/>
       <c r="I8" s="61" t="n"/>
     </row>
-    <row r="9" ht="8" customHeight="1"/>
-    <row r="10" ht="26" customHeight="1">
-      <c r="B10" s="48" t="inlineStr">
-        <is>
-          <t>Charts by Performance Band</t>
-        </is>
-      </c>
-      <c r="C10" s="54" t="n"/>
-      <c r="E10" s="48" t="inlineStr">
-        <is>
-          <t>Charts by Category</t>
-        </is>
-      </c>
-      <c r="F10" s="54" t="n"/>
-      <c r="H10" s="48" t="inlineStr">
-        <is>
-          <t>Monthly Trend — Avg Compliance %</t>
-        </is>
-      </c>
-      <c r="I10" s="53" t="n"/>
-      <c r="J10" s="54" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Band</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>Charts</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Avg %</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Excellent</t>
-        </is>
-      </c>
-      <c r="C12" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Excellent"))</f>
-        <v/>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Diabetes</t>
-        </is>
-      </c>
-      <c r="F12" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Diabetes"))</f>
-        <v/>
-      </c>
-      <c r="H12" s="9">
-        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1,1),"mmm yyyy")</f>
-        <v/>
-      </c>
-      <c r="I12" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
-        <v/>
-      </c>
-      <c r="J12" s="37">
-        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+1))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Meets Expectations</t>
-        </is>
-      </c>
-      <c r="C13" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Meets Expectations"))</f>
-        <v/>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Chronic Kidney Disease</t>
-        </is>
-      </c>
-      <c r="F13" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Chronic Kidney Disease"))</f>
-        <v/>
-      </c>
-      <c r="H13" s="9">
-        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2,1),"mmm yyyy")</f>
-        <v/>
-      </c>
-      <c r="I13" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
-        <v/>
-      </c>
-      <c r="J13" s="37">
-        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+2))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Needs Improvement</t>
-        </is>
-      </c>
-      <c r="C14" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Needs Improvement"))</f>
-        <v/>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Annual Wellness Visit</t>
-        </is>
-      </c>
-      <c r="F14" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Annual Wellness Visit"))</f>
-        <v/>
-      </c>
-      <c r="H14" s="9">
-        <f>TEXT(DATE($E$4,(MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3,1),"mmm yyyy")</f>
-        <v/>
-      </c>
-      <c r="I14" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4))</f>
-        <v/>
-      </c>
-      <c r="J14" s="37">
-        <f>IFERROR(SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3+3))*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Corrective Education Required</t>
-        </is>
-      </c>
-      <c r="C15" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$G$5:$G$200="Corrective Education Required"))</f>
-        <v/>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>High RAF Patient</t>
-        </is>
-      </c>
-      <c r="F15" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="High RAF Patient"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Random Selection</t>
-        </is>
-      </c>
-      <c r="F16" s="33">
-        <f>SUMPRODUCT(('Audit Log'!$A$5:$A$200&lt;&gt;"")*(MONTH('Audit Log'!$A$5:$A$200)&gt;=((MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)-1)*3)+1)*(MONTH('Audit Log'!$A$5:$A$200)&lt;=MATCH($C$4,{"Q1","Q2","Q3","Q4"},0)*3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$E$5:$E$200="Random Selection"))</f>
+    <row r="9" ht="10" customHeight="1">
+      <c r="A9" s="62" t="n"/>
+      <c r="B9" s="62" t="n"/>
+      <c r="C9" s="62" t="n"/>
+      <c r="D9" s="62" t="n"/>
+      <c r="E9" s="62" t="n"/>
+      <c r="F9" s="62" t="n"/>
+      <c r="G9" s="62" t="n"/>
+      <c r="H9" s="62" t="n"/>
+      <c r="I9" s="62" t="n"/>
+      <c r="J9" s="62" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Provider Progression — Monthly Compliance % by Provider</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="64" t="inlineStr">
+        <is>
+          <t>Type each provider's name in column B — the row fills in automatically from the Audit Log for the year picked above. Rising lines = improvement · falling lines = decline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="6" t="inlineStr"/>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="66" t="inlineStr">
+        <is>
+          <t>Dr. Rivera</t>
+        </is>
+      </c>
+      <c r="C13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="D13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="E13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="F13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="G13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="H13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="I13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="J13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="K13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="L13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="N13" s="67">
+        <f>IF($B13="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B13)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="65" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="66" t="inlineStr">
+        <is>
+          <t>Dr. Colón</t>
+        </is>
+      </c>
+      <c r="C14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="D14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="E14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="F14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="G14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="H14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="I14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="J14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="K14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="L14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="M14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="N14" s="67">
+        <f>IF($B14="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B14)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="65" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="66" t="n"/>
+      <c r="C15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="D15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="E15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="F15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="G15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="H15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="I15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="J15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="K15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="L15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="M15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="N15" s="67">
+        <f>IF($B15="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B15)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="65" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="66" t="n"/>
+      <c r="C16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="D16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="E16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="F16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="G16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="H16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="I16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="J16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="K16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="L16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="M16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="N16" s="67">
+        <f>IF($B16="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B16)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="65" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="66" t="n"/>
+      <c r="C17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=1)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="D17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=2)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="E17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=3)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="F17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=4)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="G17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=5)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="H17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=6)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="I17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=7)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="J17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=8)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="K17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=9)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="L17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=10)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="M17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=11)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
+        <v/>
+      </c>
+      <c r="N17" s="67">
+        <f>IF($B17="","",IFERROR(SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*'Audit Log'!$F$5:$F$200)/SUMPRODUCT(('Audit Log'!$B$5:$B$200=$B17)*ISNUMBER('Audit Log'!$A$5:$A$200)*(MONTH('Audit Log'!$A$5:$A$200)=12)*(YEAR('Audit Log'!$A$5:$A$200)=$E$4)*('Audit Log'!$F$5:$F$200&lt;&gt;"")),""))</f>
         <v/>
       </c>
     </row>
@@ -5806,21 +5877,33 @@
     <row r="53" ht="18" customHeight="1"/>
     <row r="54" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="H10:J10"/>
     <mergeCell ref="H6:I6"/>
+    <mergeCell ref="A10:N10"/>
     <mergeCell ref="D7:E8"/>
     <mergeCell ref="B7:C8"/>
-    <mergeCell ref="E10:F10"/>
     <mergeCell ref="H7:I8"/>
     <mergeCell ref="F7:G8"/>
-    <mergeCell ref="B10:C10"/>
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="A11:N11"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
+  <conditionalFormatting sqref="C13:N17">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Q1,Q2,Q3,Q4"</formula1>

</xml_diff>

<commit_message>
Add Monthly Batch (10) tab for auditing 10 claims side by side
New tab lets a single auditor complete all 10 monthly audits in one place
without duplicating tabs. Each of the 10 chart columns has its own header
(provider / claim # / DOS / category / payer), 18 rating cells, section
subtotals, weighted Overall Compliance %, and Performance Band — all
auto-computed and color-coded.

At the bottom, a Batch Summary block gives the global metrics across the
10 claims: claims audited, average compliance %, number scoring Meets+,
and number needing Corrective. Nothing overwrites between charts.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Audit Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Audit Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Quick Reference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Quarterly Report" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Batch (10)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Reference" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Report" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -378,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -559,6 +560,45 @@
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -666,13 +706,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -695,7 +735,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -703,7 +743,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -728,7 +768,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -736,7 +776,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -761,7 +801,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -769,7 +809,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -794,7 +834,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -802,7 +842,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -827,7 +867,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -835,7 +875,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -860,7 +900,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -868,7 +908,7 @@
             <symbol val="circle"/>
             <size val="7"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -913,8 +953,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -942,7 +982,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -957,9 +997,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1991,6 +2031,1166 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00B45309"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>Monthly Batch — Audit up to 10 Claims Side by Side</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="69" t="inlineStr">
+        <is>
+          <t>One column per claim · fill in the yellow header + ratings · each column's Compliance % and Rating compute automatically. Nothing gets erased between charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B4" s="70" t="n"/>
+      <c r="C4" s="70" t="n"/>
+      <c r="D4" s="70" t="n"/>
+      <c r="E4" s="70" t="n"/>
+      <c r="F4" s="70" t="n"/>
+      <c r="G4" s="70" t="n"/>
+      <c r="H4" s="70" t="n"/>
+      <c r="I4" s="70" t="n"/>
+      <c r="J4" s="70" t="n"/>
+      <c r="K4" s="70" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Claim Number</t>
+        </is>
+      </c>
+      <c r="B5" s="70" t="n"/>
+      <c r="C5" s="70" t="n"/>
+      <c r="D5" s="70" t="n"/>
+      <c r="E5" s="70" t="n"/>
+      <c r="F5" s="70" t="n"/>
+      <c r="G5" s="70" t="n"/>
+      <c r="H5" s="70" t="n"/>
+      <c r="I5" s="70" t="n"/>
+      <c r="J5" s="70" t="n"/>
+      <c r="K5" s="70" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Date of Service</t>
+        </is>
+      </c>
+      <c r="B6" s="70" t="n"/>
+      <c r="C6" s="70" t="n"/>
+      <c r="D6" s="70" t="n"/>
+      <c r="E6" s="70" t="n"/>
+      <c r="F6" s="70" t="n"/>
+      <c r="G6" s="70" t="n"/>
+      <c r="H6" s="70" t="n"/>
+      <c r="I6" s="70" t="n"/>
+      <c r="J6" s="70" t="n"/>
+      <c r="K6" s="70" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="n"/>
+      <c r="C7" s="70" t="n"/>
+      <c r="D7" s="70" t="n"/>
+      <c r="E7" s="70" t="n"/>
+      <c r="F7" s="70" t="n"/>
+      <c r="G7" s="70" t="n"/>
+      <c r="H7" s="70" t="n"/>
+      <c r="I7" s="70" t="n"/>
+      <c r="J7" s="70" t="n"/>
+      <c r="K7" s="70" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Payer</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="n"/>
+      <c r="C8" s="70" t="n"/>
+      <c r="D8" s="70" t="n"/>
+      <c r="E8" s="70" t="n"/>
+      <c r="F8" s="70" t="n"/>
+      <c r="G8" s="70" t="n"/>
+      <c r="H8" s="70" t="n"/>
+      <c r="I8" s="70" t="n"/>
+      <c r="J8" s="70" t="n"/>
+      <c r="K8" s="70" t="n"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="71" t="inlineStr">
+        <is>
+          <t>Element ↓  ·  Chart →</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>#9</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A · Diagnosis Accuracy   (30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>A1 — Diagnoses clinically supported</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="74" t="n"/>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="74" t="n"/>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="74" t="n"/>
+      <c r="J11" s="74" t="n"/>
+      <c r="K11" s="74" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="73" t="inlineStr">
+        <is>
+          <t>A2 — Chronic conditions actively addressed</t>
+        </is>
+      </c>
+      <c r="B12" s="74" t="n"/>
+      <c r="C12" s="74" t="n"/>
+      <c r="D12" s="74" t="n"/>
+      <c r="E12" s="74" t="n"/>
+      <c r="F12" s="74" t="n"/>
+      <c r="G12" s="74" t="n"/>
+      <c r="H12" s="74" t="n"/>
+      <c r="I12" s="74" t="n"/>
+      <c r="J12" s="74" t="n"/>
+      <c r="K12" s="74" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="73" t="inlineStr">
+        <is>
+          <t>A3 — No unsupported / resolved dx billed</t>
+        </is>
+      </c>
+      <c r="B13" s="74" t="n"/>
+      <c r="C13" s="74" t="n"/>
+      <c r="D13" s="74" t="n"/>
+      <c r="E13" s="74" t="n"/>
+      <c r="F13" s="74" t="n"/>
+      <c r="G13" s="74" t="n"/>
+      <c r="H13" s="74" t="n"/>
+      <c r="I13" s="74" t="n"/>
+      <c r="J13" s="74" t="n"/>
+      <c r="K13" s="74" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="73" t="inlineStr">
+        <is>
+          <t>A4 — Problem list matches A&amp;P</t>
+        </is>
+      </c>
+      <c r="B14" s="74" t="n"/>
+      <c r="C14" s="74" t="n"/>
+      <c r="D14" s="74" t="n"/>
+      <c r="E14" s="74" t="n"/>
+      <c r="F14" s="74" t="n"/>
+      <c r="G14" s="74" t="n"/>
+      <c r="H14" s="74" t="n"/>
+      <c r="I14" s="74" t="n"/>
+      <c r="J14" s="74" t="n"/>
+      <c r="K14" s="74" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B · Documentation Specificity   (25%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="73" t="inlineStr">
+        <is>
+          <t>B1 — ICD-10 at highest specificity</t>
+        </is>
+      </c>
+      <c r="B16" s="74" t="n"/>
+      <c r="C16" s="74" t="n"/>
+      <c r="D16" s="74" t="n"/>
+      <c r="E16" s="74" t="n"/>
+      <c r="F16" s="74" t="n"/>
+      <c r="G16" s="74" t="n"/>
+      <c r="H16" s="74" t="n"/>
+      <c r="I16" s="74" t="n"/>
+      <c r="J16" s="74" t="n"/>
+      <c r="K16" s="74" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="73" t="inlineStr">
+        <is>
+          <t>B2 — Diabetes: type + complications + control</t>
+        </is>
+      </c>
+      <c r="B17" s="74" t="n"/>
+      <c r="C17" s="74" t="n"/>
+      <c r="D17" s="74" t="n"/>
+      <c r="E17" s="74" t="n"/>
+      <c r="F17" s="74" t="n"/>
+      <c r="G17" s="74" t="n"/>
+      <c r="H17" s="74" t="n"/>
+      <c r="I17" s="74" t="n"/>
+      <c r="J17" s="74" t="n"/>
+      <c r="K17" s="74" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="73" t="inlineStr">
+        <is>
+          <t>B3 — S/O/A/P tell one consistent story</t>
+        </is>
+      </c>
+      <c r="B18" s="74" t="n"/>
+      <c r="C18" s="74" t="n"/>
+      <c r="D18" s="74" t="n"/>
+      <c r="E18" s="74" t="n"/>
+      <c r="F18" s="74" t="n"/>
+      <c r="G18" s="74" t="n"/>
+      <c r="H18" s="74" t="n"/>
+      <c r="I18" s="74" t="n"/>
+      <c r="J18" s="74" t="n"/>
+      <c r="K18" s="74" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="73" t="inlineStr">
+        <is>
+          <t>B4 — Note signed / dated / closed</t>
+        </is>
+      </c>
+      <c r="B19" s="74" t="n"/>
+      <c r="C19" s="74" t="n"/>
+      <c r="D19" s="74" t="n"/>
+      <c r="E19" s="74" t="n"/>
+      <c r="F19" s="74" t="n"/>
+      <c r="G19" s="74" t="n"/>
+      <c r="H19" s="74" t="n"/>
+      <c r="I19" s="74" t="n"/>
+      <c r="J19" s="74" t="n"/>
+      <c r="K19" s="74" t="n"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C · SOAP Note Structure   (25%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="73" t="inlineStr">
+        <is>
+          <t>C1 — Subjective documented</t>
+        </is>
+      </c>
+      <c r="B21" s="74" t="n"/>
+      <c r="C21" s="74" t="n"/>
+      <c r="D21" s="74" t="n"/>
+      <c r="E21" s="74" t="n"/>
+      <c r="F21" s="74" t="n"/>
+      <c r="G21" s="74" t="n"/>
+      <c r="H21" s="74" t="n"/>
+      <c r="I21" s="74" t="n"/>
+      <c r="J21" s="74" t="n"/>
+      <c r="K21" s="74" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="73" t="inlineStr">
+        <is>
+          <t>C2 — Objective documented</t>
+        </is>
+      </c>
+      <c r="B22" s="74" t="n"/>
+      <c r="C22" s="74" t="n"/>
+      <c r="D22" s="74" t="n"/>
+      <c r="E22" s="74" t="n"/>
+      <c r="F22" s="74" t="n"/>
+      <c r="G22" s="74" t="n"/>
+      <c r="H22" s="74" t="n"/>
+      <c r="I22" s="74" t="n"/>
+      <c r="J22" s="74" t="n"/>
+      <c r="K22" s="74" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="73" t="inlineStr">
+        <is>
+          <t>C3 — Assessment (dx with reasoning)</t>
+        </is>
+      </c>
+      <c r="B23" s="74" t="n"/>
+      <c r="C23" s="74" t="n"/>
+      <c r="D23" s="74" t="n"/>
+      <c r="E23" s="74" t="n"/>
+      <c r="F23" s="74" t="n"/>
+      <c r="G23" s="74" t="n"/>
+      <c r="H23" s="74" t="n"/>
+      <c r="I23" s="74" t="n"/>
+      <c r="J23" s="74" t="n"/>
+      <c r="K23" s="74" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="73" t="inlineStr">
+        <is>
+          <t>C4 — Plan documented</t>
+        </is>
+      </c>
+      <c r="B24" s="74" t="n"/>
+      <c r="C24" s="74" t="n"/>
+      <c r="D24" s="74" t="n"/>
+      <c r="E24" s="74" t="n"/>
+      <c r="F24" s="74" t="n"/>
+      <c r="G24" s="74" t="n"/>
+      <c r="H24" s="74" t="n"/>
+      <c r="I24" s="74" t="n"/>
+      <c r="J24" s="74" t="n"/>
+      <c r="K24" s="74" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D · HCC Capture   (10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="73" t="inlineStr">
+        <is>
+          <t>D1 — Prior-year HCCs recaptured</t>
+        </is>
+      </c>
+      <c r="B26" s="74" t="n"/>
+      <c r="C26" s="74" t="n"/>
+      <c r="D26" s="74" t="n"/>
+      <c r="E26" s="74" t="n"/>
+      <c r="F26" s="74" t="n"/>
+      <c r="G26" s="74" t="n"/>
+      <c r="H26" s="74" t="n"/>
+      <c r="I26" s="74" t="n"/>
+      <c r="J26" s="74" t="n"/>
+      <c r="K26" s="74" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="73" t="inlineStr">
+        <is>
+          <t>D2 — Suspected chronic conditions captured</t>
+        </is>
+      </c>
+      <c r="B27" s="74" t="n"/>
+      <c r="C27" s="74" t="n"/>
+      <c r="D27" s="74" t="n"/>
+      <c r="E27" s="74" t="n"/>
+      <c r="F27" s="74" t="n"/>
+      <c r="G27" s="74" t="n"/>
+      <c r="H27" s="74" t="n"/>
+      <c r="I27" s="74" t="n"/>
+      <c r="J27" s="74" t="n"/>
+      <c r="K27" s="74" t="n"/>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E · Documentation Supporting Quality Measures   (10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="73" t="inlineStr">
+        <is>
+          <t>E1 — Screening values documented (score/number)</t>
+        </is>
+      </c>
+      <c r="B29" s="74" t="n"/>
+      <c r="C29" s="74" t="n"/>
+      <c r="D29" s="74" t="n"/>
+      <c r="E29" s="74" t="n"/>
+      <c r="F29" s="74" t="n"/>
+      <c r="G29" s="74" t="n"/>
+      <c r="H29" s="74" t="n"/>
+      <c r="I29" s="74" t="n"/>
+      <c r="J29" s="74" t="n"/>
+      <c r="K29" s="74" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="73" t="inlineStr">
+        <is>
+          <t>E2 — Follow-up plan when positive/abnormal</t>
+        </is>
+      </c>
+      <c r="B30" s="74" t="n"/>
+      <c r="C30" s="74" t="n"/>
+      <c r="D30" s="74" t="n"/>
+      <c r="E30" s="74" t="n"/>
+      <c r="F30" s="74" t="n"/>
+      <c r="G30" s="74" t="n"/>
+      <c r="H30" s="74" t="n"/>
+      <c r="I30" s="74" t="n"/>
+      <c r="J30" s="74" t="n"/>
+      <c r="K30" s="74" t="n"/>
+    </row>
+    <row r="32" ht="6" customHeight="1"/>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="75" t="inlineStr">
+        <is>
+          <t>SECTION SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="17" t="n"/>
+      <c r="I33" s="17" t="n"/>
+      <c r="J33" s="17" t="n"/>
+      <c r="K33" s="17" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A · % Met  (weight 30%)</t>
+        </is>
+      </c>
+      <c r="B34" s="76">
+        <f>IFERROR((COUNTIF(B11:B14,"✓")+COUNTIF(B11:B14,"△")*0.5)/(COUNTIF(B11:B14,"✓")+COUNTIF(B11:B14,"△")+COUNTIF(B11:B14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="C34" s="76">
+        <f>IFERROR((COUNTIF(C11:C14,"✓")+COUNTIF(C11:C14,"△")*0.5)/(COUNTIF(C11:C14,"✓")+COUNTIF(C11:C14,"△")+COUNTIF(C11:C14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="D34" s="76">
+        <f>IFERROR((COUNTIF(D11:D14,"✓")+COUNTIF(D11:D14,"△")*0.5)/(COUNTIF(D11:D14,"✓")+COUNTIF(D11:D14,"△")+COUNTIF(D11:D14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="76">
+        <f>IFERROR((COUNTIF(E11:E14,"✓")+COUNTIF(E11:E14,"△")*0.5)/(COUNTIF(E11:E14,"✓")+COUNTIF(E11:E14,"△")+COUNTIF(E11:E14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="76">
+        <f>IFERROR((COUNTIF(F11:F14,"✓")+COUNTIF(F11:F14,"△")*0.5)/(COUNTIF(F11:F14,"✓")+COUNTIF(F11:F14,"△")+COUNTIF(F11:F14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="76">
+        <f>IFERROR((COUNTIF(G11:G14,"✓")+COUNTIF(G11:G14,"△")*0.5)/(COUNTIF(G11:G14,"✓")+COUNTIF(G11:G14,"△")+COUNTIF(G11:G14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="76">
+        <f>IFERROR((COUNTIF(H11:H14,"✓")+COUNTIF(H11:H14,"△")*0.5)/(COUNTIF(H11:H14,"✓")+COUNTIF(H11:H14,"△")+COUNTIF(H11:H14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="76">
+        <f>IFERROR((COUNTIF(I11:I14,"✓")+COUNTIF(I11:I14,"△")*0.5)/(COUNTIF(I11:I14,"✓")+COUNTIF(I11:I14,"△")+COUNTIF(I11:I14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="76">
+        <f>IFERROR((COUNTIF(J11:J14,"✓")+COUNTIF(J11:J14,"△")*0.5)/(COUNTIF(J11:J14,"✓")+COUNTIF(J11:J14,"△")+COUNTIF(J11:J14,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="76">
+        <f>IFERROR((COUNTIF(K11:K14,"✓")+COUNTIF(K11:K14,"△")*0.5)/(COUNTIF(K11:K14,"✓")+COUNTIF(K11:K14,"△")+COUNTIF(K11:K14,"✗")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B · % Met  (weight 25%)</t>
+        </is>
+      </c>
+      <c r="B35" s="76">
+        <f>IFERROR((COUNTIF(B16:B19,"✓")+COUNTIF(B16:B19,"△")*0.5)/(COUNTIF(B16:B19,"✓")+COUNTIF(B16:B19,"△")+COUNTIF(B16:B19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="C35" s="76">
+        <f>IFERROR((COUNTIF(C16:C19,"✓")+COUNTIF(C16:C19,"△")*0.5)/(COUNTIF(C16:C19,"✓")+COUNTIF(C16:C19,"△")+COUNTIF(C16:C19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="D35" s="76">
+        <f>IFERROR((COUNTIF(D16:D19,"✓")+COUNTIF(D16:D19,"△")*0.5)/(COUNTIF(D16:D19,"✓")+COUNTIF(D16:D19,"△")+COUNTIF(D16:D19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="76">
+        <f>IFERROR((COUNTIF(E16:E19,"✓")+COUNTIF(E16:E19,"△")*0.5)/(COUNTIF(E16:E19,"✓")+COUNTIF(E16:E19,"△")+COUNTIF(E16:E19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="76">
+        <f>IFERROR((COUNTIF(F16:F19,"✓")+COUNTIF(F16:F19,"△")*0.5)/(COUNTIF(F16:F19,"✓")+COUNTIF(F16:F19,"△")+COUNTIF(F16:F19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="76">
+        <f>IFERROR((COUNTIF(G16:G19,"✓")+COUNTIF(G16:G19,"△")*0.5)/(COUNTIF(G16:G19,"✓")+COUNTIF(G16:G19,"△")+COUNTIF(G16:G19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="76">
+        <f>IFERROR((COUNTIF(H16:H19,"✓")+COUNTIF(H16:H19,"△")*0.5)/(COUNTIF(H16:H19,"✓")+COUNTIF(H16:H19,"△")+COUNTIF(H16:H19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="76">
+        <f>IFERROR((COUNTIF(I16:I19,"✓")+COUNTIF(I16:I19,"△")*0.5)/(COUNTIF(I16:I19,"✓")+COUNTIF(I16:I19,"△")+COUNTIF(I16:I19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="76">
+        <f>IFERROR((COUNTIF(J16:J19,"✓")+COUNTIF(J16:J19,"△")*0.5)/(COUNTIF(J16:J19,"✓")+COUNTIF(J16:J19,"△")+COUNTIF(J16:J19,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="76">
+        <f>IFERROR((COUNTIF(K16:K19,"✓")+COUNTIF(K16:K19,"△")*0.5)/(COUNTIF(K16:K19,"✓")+COUNTIF(K16:K19,"△")+COUNTIF(K16:K19,"✗")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C · % Met  (weight 25%)</t>
+        </is>
+      </c>
+      <c r="B36" s="76">
+        <f>IFERROR((COUNTIF(B21:B24,"✓")+COUNTIF(B21:B24,"△")*0.5)/(COUNTIF(B21:B24,"✓")+COUNTIF(B21:B24,"△")+COUNTIF(B21:B24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="C36" s="76">
+        <f>IFERROR((COUNTIF(C21:C24,"✓")+COUNTIF(C21:C24,"△")*0.5)/(COUNTIF(C21:C24,"✓")+COUNTIF(C21:C24,"△")+COUNTIF(C21:C24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="D36" s="76">
+        <f>IFERROR((COUNTIF(D21:D24,"✓")+COUNTIF(D21:D24,"△")*0.5)/(COUNTIF(D21:D24,"✓")+COUNTIF(D21:D24,"△")+COUNTIF(D21:D24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="76">
+        <f>IFERROR((COUNTIF(E21:E24,"✓")+COUNTIF(E21:E24,"△")*0.5)/(COUNTIF(E21:E24,"✓")+COUNTIF(E21:E24,"△")+COUNTIF(E21:E24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="76">
+        <f>IFERROR((COUNTIF(F21:F24,"✓")+COUNTIF(F21:F24,"△")*0.5)/(COUNTIF(F21:F24,"✓")+COUNTIF(F21:F24,"△")+COUNTIF(F21:F24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="76">
+        <f>IFERROR((COUNTIF(G21:G24,"✓")+COUNTIF(G21:G24,"△")*0.5)/(COUNTIF(G21:G24,"✓")+COUNTIF(G21:G24,"△")+COUNTIF(G21:G24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="76">
+        <f>IFERROR((COUNTIF(H21:H24,"✓")+COUNTIF(H21:H24,"△")*0.5)/(COUNTIF(H21:H24,"✓")+COUNTIF(H21:H24,"△")+COUNTIF(H21:H24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="76">
+        <f>IFERROR((COUNTIF(I21:I24,"✓")+COUNTIF(I21:I24,"△")*0.5)/(COUNTIF(I21:I24,"✓")+COUNTIF(I21:I24,"△")+COUNTIF(I21:I24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="76">
+        <f>IFERROR((COUNTIF(J21:J24,"✓")+COUNTIF(J21:J24,"△")*0.5)/(COUNTIF(J21:J24,"✓")+COUNTIF(J21:J24,"△")+COUNTIF(J21:J24,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="K36" s="76">
+        <f>IFERROR((COUNTIF(K21:K24,"✓")+COUNTIF(K21:K24,"△")*0.5)/(COUNTIF(K21:K24,"✓")+COUNTIF(K21:K24,"△")+COUNTIF(K21:K24,"✗")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D · % Met  (weight 10%)</t>
+        </is>
+      </c>
+      <c r="B37" s="76">
+        <f>IFERROR((COUNTIF(B26:B27,"✓")+COUNTIF(B26:B27,"△")*0.5)/(COUNTIF(B26:B27,"✓")+COUNTIF(B26:B27,"△")+COUNTIF(B26:B27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="C37" s="76">
+        <f>IFERROR((COUNTIF(C26:C27,"✓")+COUNTIF(C26:C27,"△")*0.5)/(COUNTIF(C26:C27,"✓")+COUNTIF(C26:C27,"△")+COUNTIF(C26:C27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="D37" s="76">
+        <f>IFERROR((COUNTIF(D26:D27,"✓")+COUNTIF(D26:D27,"△")*0.5)/(COUNTIF(D26:D27,"✓")+COUNTIF(D26:D27,"△")+COUNTIF(D26:D27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="76">
+        <f>IFERROR((COUNTIF(E26:E27,"✓")+COUNTIF(E26:E27,"△")*0.5)/(COUNTIF(E26:E27,"✓")+COUNTIF(E26:E27,"△")+COUNTIF(E26:E27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="76">
+        <f>IFERROR((COUNTIF(F26:F27,"✓")+COUNTIF(F26:F27,"△")*0.5)/(COUNTIF(F26:F27,"✓")+COUNTIF(F26:F27,"△")+COUNTIF(F26:F27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="76">
+        <f>IFERROR((COUNTIF(G26:G27,"✓")+COUNTIF(G26:G27,"△")*0.5)/(COUNTIF(G26:G27,"✓")+COUNTIF(G26:G27,"△")+COUNTIF(G26:G27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="76">
+        <f>IFERROR((COUNTIF(H26:H27,"✓")+COUNTIF(H26:H27,"△")*0.5)/(COUNTIF(H26:H27,"✓")+COUNTIF(H26:H27,"△")+COUNTIF(H26:H27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="76">
+        <f>IFERROR((COUNTIF(I26:I27,"✓")+COUNTIF(I26:I27,"△")*0.5)/(COUNTIF(I26:I27,"✓")+COUNTIF(I26:I27,"△")+COUNTIF(I26:I27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="76">
+        <f>IFERROR((COUNTIF(J26:J27,"✓")+COUNTIF(J26:J27,"△")*0.5)/(COUNTIF(J26:J27,"✓")+COUNTIF(J26:J27,"△")+COUNTIF(J26:J27,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="K37" s="76">
+        <f>IFERROR((COUNTIF(K26:K27,"✓")+COUNTIF(K26:K27,"△")*0.5)/(COUNTIF(K26:K27,"✓")+COUNTIF(K26:K27,"△")+COUNTIF(K26:K27,"✗")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E · % Met  (weight 10%)</t>
+        </is>
+      </c>
+      <c r="B38" s="76">
+        <f>IFERROR((COUNTIF(B29:B30,"✓")+COUNTIF(B29:B30,"△")*0.5)/(COUNTIF(B29:B30,"✓")+COUNTIF(B29:B30,"△")+COUNTIF(B29:B30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="C38" s="76">
+        <f>IFERROR((COUNTIF(C29:C30,"✓")+COUNTIF(C29:C30,"△")*0.5)/(COUNTIF(C29:C30,"✓")+COUNTIF(C29:C30,"△")+COUNTIF(C29:C30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="76">
+        <f>IFERROR((COUNTIF(D29:D30,"✓")+COUNTIF(D29:D30,"△")*0.5)/(COUNTIF(D29:D30,"✓")+COUNTIF(D29:D30,"△")+COUNTIF(D29:D30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="76">
+        <f>IFERROR((COUNTIF(E29:E30,"✓")+COUNTIF(E29:E30,"△")*0.5)/(COUNTIF(E29:E30,"✓")+COUNTIF(E29:E30,"△")+COUNTIF(E29:E30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="76">
+        <f>IFERROR((COUNTIF(F29:F30,"✓")+COUNTIF(F29:F30,"△")*0.5)/(COUNTIF(F29:F30,"✓")+COUNTIF(F29:F30,"△")+COUNTIF(F29:F30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="76">
+        <f>IFERROR((COUNTIF(G29:G30,"✓")+COUNTIF(G29:G30,"△")*0.5)/(COUNTIF(G29:G30,"✓")+COUNTIF(G29:G30,"△")+COUNTIF(G29:G30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="76">
+        <f>IFERROR((COUNTIF(H29:H30,"✓")+COUNTIF(H29:H30,"△")*0.5)/(COUNTIF(H29:H30,"✓")+COUNTIF(H29:H30,"△")+COUNTIF(H29:H30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="76">
+        <f>IFERROR((COUNTIF(I29:I30,"✓")+COUNTIF(I29:I30,"△")*0.5)/(COUNTIF(I29:I30,"✓")+COUNTIF(I29:I30,"△")+COUNTIF(I29:I30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="76">
+        <f>IFERROR((COUNTIF(J29:J30,"✓")+COUNTIF(J29:J30,"△")*0.5)/(COUNTIF(J29:J30,"✓")+COUNTIF(J29:J30,"△")+COUNTIF(J29:J30,"✗")),"")</f>
+        <v/>
+      </c>
+      <c r="K38" s="76">
+        <f>IFERROR((COUNTIF(K29:K30,"✓")+COUNTIF(K29:K30,"△")*0.5)/(COUNTIF(K29:K30,"✓")+COUNTIF(K29:K30,"△")+COUNTIF(K29:K30,"✗")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>OVERALL COMPLIANCE %</t>
+        </is>
+      </c>
+      <c r="B40" s="77">
+        <f>IFERROR((IFERROR(B34,0)*IF(B34="",0,0.3)+IFERROR(B35,0)*IF(B35="",0,0.25)+IFERROR(B36,0)*IF(B36="",0,0.25)+IFERROR(B37,0)*IF(B37="",0,0.1)+IFERROR(B38,0)*IF(B38="",0,0.1))/(IF(B34="",0,0.3)+IF(B35="",0,0.25)+IF(B36="",0,0.25)+IF(B37="",0,0.1)+IF(B38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="C40" s="77">
+        <f>IFERROR((IFERROR(C34,0)*IF(C34="",0,0.3)+IFERROR(C35,0)*IF(C35="",0,0.25)+IFERROR(C36,0)*IF(C36="",0,0.25)+IFERROR(C37,0)*IF(C37="",0,0.1)+IFERROR(C38,0)*IF(C38="",0,0.1))/(IF(C34="",0,0.3)+IF(C35="",0,0.25)+IF(C36="",0,0.25)+IF(C37="",0,0.1)+IF(C38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="D40" s="77">
+        <f>IFERROR((IFERROR(D34,0)*IF(D34="",0,0.3)+IFERROR(D35,0)*IF(D35="",0,0.25)+IFERROR(D36,0)*IF(D36="",0,0.25)+IFERROR(D37,0)*IF(D37="",0,0.1)+IFERROR(D38,0)*IF(D38="",0,0.1))/(IF(D34="",0,0.3)+IF(D35="",0,0.25)+IF(D36="",0,0.25)+IF(D37="",0,0.1)+IF(D38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="77">
+        <f>IFERROR((IFERROR(E34,0)*IF(E34="",0,0.3)+IFERROR(E35,0)*IF(E35="",0,0.25)+IFERROR(E36,0)*IF(E36="",0,0.25)+IFERROR(E37,0)*IF(E37="",0,0.1)+IFERROR(E38,0)*IF(E38="",0,0.1))/(IF(E34="",0,0.3)+IF(E35="",0,0.25)+IF(E36="",0,0.25)+IF(E37="",0,0.1)+IF(E38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="77">
+        <f>IFERROR((IFERROR(F34,0)*IF(F34="",0,0.3)+IFERROR(F35,0)*IF(F35="",0,0.25)+IFERROR(F36,0)*IF(F36="",0,0.25)+IFERROR(F37,0)*IF(F37="",0,0.1)+IFERROR(F38,0)*IF(F38="",0,0.1))/(IF(F34="",0,0.3)+IF(F35="",0,0.25)+IF(F36="",0,0.25)+IF(F37="",0,0.1)+IF(F38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="77">
+        <f>IFERROR((IFERROR(G34,0)*IF(G34="",0,0.3)+IFERROR(G35,0)*IF(G35="",0,0.25)+IFERROR(G36,0)*IF(G36="",0,0.25)+IFERROR(G37,0)*IF(G37="",0,0.1)+IFERROR(G38,0)*IF(G38="",0,0.1))/(IF(G34="",0,0.3)+IF(G35="",0,0.25)+IF(G36="",0,0.25)+IF(G37="",0,0.1)+IF(G38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="77">
+        <f>IFERROR((IFERROR(H34,0)*IF(H34="",0,0.3)+IFERROR(H35,0)*IF(H35="",0,0.25)+IFERROR(H36,0)*IF(H36="",0,0.25)+IFERROR(H37,0)*IF(H37="",0,0.1)+IFERROR(H38,0)*IF(H38="",0,0.1))/(IF(H34="",0,0.3)+IF(H35="",0,0.25)+IF(H36="",0,0.25)+IF(H37="",0,0.1)+IF(H38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="77">
+        <f>IFERROR((IFERROR(I34,0)*IF(I34="",0,0.3)+IFERROR(I35,0)*IF(I35="",0,0.25)+IFERROR(I36,0)*IF(I36="",0,0.25)+IFERROR(I37,0)*IF(I37="",0,0.1)+IFERROR(I38,0)*IF(I38="",0,0.1))/(IF(I34="",0,0.3)+IF(I35="",0,0.25)+IF(I36="",0,0.25)+IF(I37="",0,0.1)+IF(I38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="77">
+        <f>IFERROR((IFERROR(J34,0)*IF(J34="",0,0.3)+IFERROR(J35,0)*IF(J35="",0,0.25)+IFERROR(J36,0)*IF(J36="",0,0.25)+IFERROR(J37,0)*IF(J37="",0,0.1)+IFERROR(J38,0)*IF(J38="",0,0.1))/(IF(J34="",0,0.3)+IF(J35="",0,0.25)+IF(J36="",0,0.25)+IF(J37="",0,0.1)+IF(J38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+      <c r="K40" s="77">
+        <f>IFERROR((IFERROR(K34,0)*IF(K34="",0,0.3)+IFERROR(K35,0)*IF(K35="",0,0.25)+IFERROR(K36,0)*IF(K36="",0,0.25)+IFERROR(K37,0)*IF(K37="",0,0.1)+IFERROR(K38,0)*IF(K38="",0,0.1))/(IF(K34="",0,0.3)+IF(K35="",0,0.25)+IF(K36="",0,0.25)+IF(K37="",0,0.1)+IF(K38="",0,0.1)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="40" t="inlineStr">
+        <is>
+          <t>RATING</t>
+        </is>
+      </c>
+      <c r="B41" s="78">
+        <f>IF(B40="","",IF(B40&gt;=0.95,"Excellent",IF(B40&gt;=0.9,"Meets",IF(B40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="C41" s="78">
+        <f>IF(C40="","",IF(C40&gt;=0.95,"Excellent",IF(C40&gt;=0.9,"Meets",IF(C40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="D41" s="78">
+        <f>IF(D40="","",IF(D40&gt;=0.95,"Excellent",IF(D40&gt;=0.9,"Meets",IF(D40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="E41" s="78">
+        <f>IF(E40="","",IF(E40&gt;=0.95,"Excellent",IF(E40&gt;=0.9,"Meets",IF(E40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="F41" s="78">
+        <f>IF(F40="","",IF(F40&gt;=0.95,"Excellent",IF(F40&gt;=0.9,"Meets",IF(F40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="G41" s="78">
+        <f>IF(G40="","",IF(G40&gt;=0.95,"Excellent",IF(G40&gt;=0.9,"Meets",IF(G40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="H41" s="78">
+        <f>IF(H40="","",IF(H40&gt;=0.95,"Excellent",IF(H40&gt;=0.9,"Meets",IF(H40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="I41" s="78">
+        <f>IF(I40="","",IF(I40&gt;=0.95,"Excellent",IF(I40&gt;=0.9,"Meets",IF(I40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="J41" s="78">
+        <f>IF(J40="","",IF(J40&gt;=0.95,"Excellent",IF(J40&gt;=0.9,"Meets",IF(J40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+      <c r="K41" s="78">
+        <f>IF(K40="","",IF(K40&gt;=0.95,"Excellent",IF(K40&gt;=0.9,"Meets",IF(K40&gt;=0.8,"Needs Impr","Corrective"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="6" customHeight="1"/>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  BATCH SUMMARY (this month)</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="n"/>
+      <c r="C44" s="17" t="n"/>
+      <c r="D44" s="17" t="n"/>
+      <c r="E44" s="17" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Claims audited</t>
+        </is>
+      </c>
+      <c r="D45" s="79">
+        <f>COUNT(B40:K40)</f>
+        <v/>
+      </c>
+      <c r="E45" s="14" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Average compliance %</t>
+        </is>
+      </c>
+      <c r="D46" s="80">
+        <f>IFERROR(AVERAGE(B40:K40),"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="14" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Charts scoring Meets+ (≥90%)</t>
+        </is>
+      </c>
+      <c r="D47" s="79">
+        <f>COUNTIF(B40:K40,"&gt;=0.9")</f>
+        <v/>
+      </c>
+      <c r="E47" s="14" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Charts needing Corrective (&lt;80%)</t>
+        </is>
+      </c>
+      <c r="D48" s="79">
+        <f>COUNTIFS(B40:K40,"&lt;0.8",B40:K40,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="E48" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A10:K10"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B11:B30">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>B11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>B11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>B11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11:C30">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>C11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>C11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>C11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="3">
+      <formula>C11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11:D30">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>D11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="1">
+      <formula>D11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="2">
+      <formula>D11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="3">
+      <formula>D11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11:E30">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>E11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>E11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="2">
+      <formula>E11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="3">
+      <formula>E11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11:F30">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>F11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="1">
+      <formula>F11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19" dxfId="2">
+      <formula>F11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="3">
+      <formula>F11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:G30">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>G11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="1">
+      <formula>G11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="2">
+      <formula>G11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="3">
+      <formula>G11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11:H30">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>H11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="1">
+      <formula>H11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="2">
+      <formula>H11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="28" dxfId="3">
+      <formula>H11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I11:I30">
+    <cfRule type="expression" priority="29" dxfId="0">
+      <formula>I11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="1">
+      <formula>I11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" dxfId="2">
+      <formula>I11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="3">
+      <formula>I11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11:J30">
+    <cfRule type="expression" priority="33" dxfId="0">
+      <formula>J11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="34" dxfId="1">
+      <formula>J11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="2">
+      <formula>J11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="36" dxfId="3">
+      <formula>J11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K11:K30">
+    <cfRule type="expression" priority="37" dxfId="0">
+      <formula>K11="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="1">
+      <formula>K11="△"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="2">
+      <formula>K11="✗"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="40" dxfId="3">
+      <formula>K11="N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B34:K34">
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="42" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="43" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35:K35">
+    <cfRule type="cellIs" priority="44" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="45" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="46" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B36:K36">
+    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="48" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="49" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B37:K37">
+    <cfRule type="cellIs" priority="50" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="51" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="52" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B38:K38">
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="0">
+      <formula>0.9</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="54" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="55" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B40:K40">
+    <cfRule type="cellIs" priority="56" operator="greaterThanOrEqual" dxfId="3">
+      <formula>0.95</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="57" operator="between" dxfId="0">
+      <formula>0.9</formula>
+      <formula>0.9499</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="58" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>0.8999</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="59" operator="between" dxfId="2">
+      <formula>0.0001</formula>
+      <formula>0.7999</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B41:K41">
+    <cfRule type="expression" priority="60" dxfId="3">
+      <formula>B41="Excellent"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="61" dxfId="0">
+      <formula>B41="Meets"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="62" dxfId="1">
+      <formula>B41="Needs Impr"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="63" dxfId="2">
+      <formula>B41="Corrective"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="B7:K7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8:K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11:K30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,△,✗,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001E40AF"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -4573,7 +5773,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00334155"/>
@@ -5334,7 +6534,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B45309"/>

</xml_diff>

<commit_message>
Add 'Start a new provider' helper card
Side panel on Audit Checklist and every Claim tab now includes 5 steps
for resetting all 10 Claim tabs at once using Excel's group-sheets
feature. The Audit Log retains every prior claim's summary so switching
providers doesn't lose historical metrics.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -1348,10 +1348,14 @@
       <c r="E4" s="28" t="inlineStr">
         <is>
           <t>How to audit a claim
-1. Click a Claim 01–10 tab (bottom of the workbook)
-2. Fill the yellow header + ratings — auto-scores
-3. Log the finished claim on the Audit Log tab
-4. Move to the next Claim tab · this Audit Checklist tab stays as the master template</t>
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -2084,11 +2088,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2478,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -2602,7 +2609,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -2696,11 +2702,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3092,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -3214,7 +3223,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -7234,11 +7242,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -7620,7 +7632,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -7752,7 +7763,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -7846,11 +7856,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8246,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -8364,7 +8377,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -8458,11 +8470,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -8844,7 +8860,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -8976,7 +8991,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -9070,11 +9084,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9474,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -9588,7 +9605,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -9682,11 +9698,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -10068,7 +10088,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -10200,7 +10219,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -10294,11 +10312,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -10680,7 +10702,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -10812,7 +10833,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -10906,11 +10926,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11316,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -11424,7 +11447,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -11518,11 +11540,15 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>How to use
-1. Fill in the yellow cells at top
-2. Rate each element (dropdown in column C)
-3. Overall % + Rating appear at the bottom
-4. Log the chart on the Audit Log tab when done</t>
+          <t>How to audit a claim
+1. Click Claim 01 → fill yellow cells → next Claim tab
+2. Log each finished claim on the Audit Log
+Start a new provider (after 10 claims)
+1. Ctrl+click tabs Claim 01 through Claim 10 to group them
+2. On any grouped tab, select the yellow cells + rating column + notes
+3. Press Delete → all 10 tabs clear at once
+4. Right-click any tab → Ungroup Sheets
+5. The Audit Log keeps every prior claim's summary — nothing is lost</t>
         </is>
       </c>
     </row>
@@ -11904,7 +11930,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -12036,7 +12061,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Restore dropdowns on Claim 01-10 tabs
openpyxl's copy_worksheet does not carry data validations to the copy.
Re-add the three DVs (Category, Payer, Rating ✓/△/✗/N/A) on every Claim
tab so the pull-downs work again.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -272,7 +272,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -407,11 +407,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -699,6 +708,8 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1839,7 +1850,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -1975,7 +1985,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -2654,7 +2663,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -2786,7 +2794,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -2904,6 +2911,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -3350,7 +3368,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -3482,7 +3499,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -3600,6 +3616,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -4046,7 +4073,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -4178,7 +4204,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -4296,6 +4321,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -8487,6 +8523,7 @@
           <t>Provider (from Claim 01)</t>
         </is>
       </c>
+      <c r="C4" s="54" t="n"/>
       <c r="D4" s="88">
         <f>'Claim 01'!B4</f>
         <v/>
@@ -8500,35 +8537,37 @@
           <t>Claims completed</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n"/>
-      <c r="C6" s="45" t="n"/>
+      <c r="B6" s="53" t="n"/>
+      <c r="C6" s="54" t="n"/>
       <c r="D6" s="92" t="inlineStr">
         <is>
           <t>Average compliance %</t>
         </is>
       </c>
-      <c r="E6" s="45" t="n"/>
-      <c r="F6" s="45" t="n"/>
+      <c r="E6" s="53" t="n"/>
+      <c r="F6" s="54" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="93">
         <f>COUNT('Claim 01:Claim 10'!I44)</f>
         <v/>
       </c>
-      <c r="B7" s="94" t="n"/>
-      <c r="C7" s="94" t="n"/>
+      <c r="B7" s="107" t="n"/>
+      <c r="C7" s="59" t="n"/>
       <c r="D7" s="95">
         <f>IFERROR(AVERAGE('Claim 01:Claim 10'!I44),"")</f>
         <v/>
       </c>
-      <c r="E7" s="94" t="n"/>
-      <c r="F7" s="94" t="n"/>
+      <c r="E7" s="107" t="n"/>
+      <c r="F7" s="59" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="94" t="n"/>
-      <c r="C8" s="94" t="n"/>
-      <c r="E8" s="94" t="n"/>
-      <c r="F8" s="94" t="n"/>
+      <c r="A8" s="60" t="n"/>
+      <c r="B8" s="108" t="n"/>
+      <c r="C8" s="61" t="n"/>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="108" t="n"/>
+      <c r="F8" s="61" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="92" t="inlineStr">
@@ -8536,35 +8575,37 @@
           <t>Meeting Expectations (≥90%)</t>
         </is>
       </c>
-      <c r="B10" s="45" t="n"/>
-      <c r="C10" s="45" t="n"/>
+      <c r="B10" s="53" t="n"/>
+      <c r="C10" s="54" t="n"/>
       <c r="D10" s="92" t="inlineStr">
         <is>
           <t>Corrective Required (&lt;80%)</t>
         </is>
       </c>
-      <c r="E10" s="45" t="n"/>
-      <c r="F10" s="45" t="n"/>
+      <c r="E10" s="53" t="n"/>
+      <c r="F10" s="54" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="93">
         <f>COUNTIFS(E17:E26,"&gt;=0.9",E17:E26,"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="B11" s="94" t="n"/>
-      <c r="C11" s="94" t="n"/>
+      <c r="B11" s="107" t="n"/>
+      <c r="C11" s="59" t="n"/>
       <c r="D11" s="93">
         <f>COUNTIFS(E17:E26,"&lt;0.8",E17:E26,"&gt;0")</f>
         <v/>
       </c>
-      <c r="E11" s="94" t="n"/>
-      <c r="F11" s="94" t="n"/>
+      <c r="E11" s="107" t="n"/>
+      <c r="F11" s="59" t="n"/>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="B12" s="94" t="n"/>
-      <c r="C12" s="94" t="n"/>
-      <c r="E12" s="94" t="n"/>
-      <c r="F12" s="94" t="n"/>
+      <c r="A12" s="60" t="n"/>
+      <c r="B12" s="108" t="n"/>
+      <c r="C12" s="61" t="n"/>
+      <c r="D12" s="60" t="n"/>
+      <c r="E12" s="108" t="n"/>
+      <c r="F12" s="61" t="n"/>
     </row>
     <row r="14" ht="12" customHeight="1"/>
     <row r="15" ht="26" customHeight="1">
@@ -8862,10 +8903,14 @@
           <t xml:space="preserve">  OVERALL PROVIDER PERFORMANCE BAND</t>
         </is>
       </c>
+      <c r="B28" s="53" t="n"/>
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="54" t="n"/>
       <c r="E28" s="98">
         <f>IF(D7="","",IF(D7&gt;=0.95,"Excellent",IF(D7&gt;=0.9,"Meets Expectations",IF(D7&gt;=0.8,"Needs Improvement","Corrective Education Required"))))</f>
         <v/>
       </c>
+      <c r="F28" s="54" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="96" t="inlineStr">
@@ -8880,10 +8925,10 @@
           <t>Band</t>
         </is>
       </c>
-      <c r="B31" s="45" t="n"/>
-      <c r="C31" s="45" t="n"/>
-      <c r="D31" s="45" t="n"/>
-      <c r="E31" s="45" t="n"/>
+      <c r="B31" s="53" t="n"/>
+      <c r="C31" s="53" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="54" t="n"/>
       <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Count</t>
@@ -8896,10 +8941,10 @@
           <t>Excellent</t>
         </is>
       </c>
-      <c r="B32" s="100" t="n"/>
-      <c r="C32" s="100" t="n"/>
-      <c r="D32" s="100" t="n"/>
-      <c r="E32" s="100" t="n"/>
+      <c r="B32" s="53" t="n"/>
+      <c r="C32" s="53" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="54" t="n"/>
       <c r="F32" s="18">
         <f>COUNTIF(F17:F26,"Excellent")</f>
         <v/>
@@ -8911,10 +8956,10 @@
           <t>Meets Expectations</t>
         </is>
       </c>
-      <c r="B33" s="102" t="n"/>
-      <c r="C33" s="102" t="n"/>
-      <c r="D33" s="102" t="n"/>
-      <c r="E33" s="102" t="n"/>
+      <c r="B33" s="53" t="n"/>
+      <c r="C33" s="53" t="n"/>
+      <c r="D33" s="53" t="n"/>
+      <c r="E33" s="54" t="n"/>
       <c r="F33" s="18">
         <f>COUNTIF(F17:F26,"Meets Expectations")</f>
         <v/>
@@ -8926,10 +8971,10 @@
           <t>Needs Improvement</t>
         </is>
       </c>
-      <c r="B34" s="104" t="n"/>
-      <c r="C34" s="104" t="n"/>
-      <c r="D34" s="104" t="n"/>
-      <c r="E34" s="104" t="n"/>
+      <c r="B34" s="53" t="n"/>
+      <c r="C34" s="53" t="n"/>
+      <c r="D34" s="53" t="n"/>
+      <c r="E34" s="54" t="n"/>
       <c r="F34" s="18">
         <f>COUNTIF(F17:F26,"Needs Improvement")</f>
         <v/>
@@ -8941,10 +8986,10 @@
           <t>Corrective Education Required</t>
         </is>
       </c>
-      <c r="B35" s="106" t="n"/>
-      <c r="C35" s="106" t="n"/>
-      <c r="D35" s="106" t="n"/>
-      <c r="E35" s="106" t="n"/>
+      <c r="B35" s="53" t="n"/>
+      <c r="C35" s="53" t="n"/>
+      <c r="D35" s="53" t="n"/>
+      <c r="E35" s="54" t="n"/>
       <c r="F35" s="18">
         <f>COUNTIF(F17:F26,"Corrective Education Required")</f>
         <v/>
@@ -9480,7 +9525,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -9612,7 +9656,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -9730,6 +9773,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -10176,7 +10230,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -10308,7 +10361,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -10426,6 +10478,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -10872,7 +10935,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -11004,7 +11066,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -11122,6 +11183,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -11568,7 +11640,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -11700,7 +11771,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -11818,6 +11888,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -12264,7 +12345,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -12396,7 +12476,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -12514,6 +12593,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -12960,7 +13050,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -13092,7 +13181,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -13210,6 +13298,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
@@ -13656,7 +13755,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -13788,7 +13886,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -13906,6 +14003,17 @@
     <mergeCell ref="A9:E9"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Diabetes,Chronic Kidney Disease,Annual Wellness Visit,High RAF Patient,Random Selection"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Medicare Advantage,Commercial,Medicaid,Dual"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10:C34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓ Met,△ Partial,✗ Not Met,N/A"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Fix Provider Metrics cell references (D44/D45, not I44/I45)
Overall Compliance % and Performance Band cells on the Audit Checklist
template live in column D, not column I. Provider Metrics KPI tiles and
per-claim breakdown were reading empty cells and never updating.

Now every tile and table cell reads the correct column, so all metrics
recalculate live as ratings are ticked on any Claim tab.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -1850,6 +1850,7 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
+    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -1985,6 +1986,7 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
+    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -8549,13 +8551,13 @@
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="93">
-        <f>COUNT('Claim 01:Claim 10'!I44)</f>
+        <f>COUNT('Claim 01:Claim 10'!D44)</f>
         <v/>
       </c>
       <c r="B7" s="107" t="n"/>
       <c r="C7" s="59" t="n"/>
       <c r="D7" s="95">
-        <f>IFERROR(AVERAGE('Claim 01:Claim 10'!I44),"")</f>
+        <f>IFERROR(AVERAGE('Claim 01:Claim 10'!D44),"")</f>
         <v/>
       </c>
       <c r="E7" s="107" t="n"/>
@@ -8664,11 +8666,11 @@
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>IFERROR('Claim 01'!I44,"")</f>
+        <f>IFERROR('Claim 01'!D44,"")</f>
         <v/>
       </c>
       <c r="F17" s="9">
-        <f>IFERROR('Claim 01'!I45,"")</f>
+        <f>IFERROR('Claim 01'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8689,11 +8691,11 @@
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>IFERROR('Claim 02'!I44,"")</f>
+        <f>IFERROR('Claim 02'!D44,"")</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>IFERROR('Claim 02'!I45,"")</f>
+        <f>IFERROR('Claim 02'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8714,11 +8716,11 @@
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>IFERROR('Claim 03'!I44,"")</f>
+        <f>IFERROR('Claim 03'!D44,"")</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>IFERROR('Claim 03'!I45,"")</f>
+        <f>IFERROR('Claim 03'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8739,11 +8741,11 @@
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>IFERROR('Claim 04'!I44,"")</f>
+        <f>IFERROR('Claim 04'!D44,"")</f>
         <v/>
       </c>
       <c r="F20" s="9">
-        <f>IFERROR('Claim 04'!I45,"")</f>
+        <f>IFERROR('Claim 04'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8764,11 +8766,11 @@
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>IFERROR('Claim 05'!I44,"")</f>
+        <f>IFERROR('Claim 05'!D44,"")</f>
         <v/>
       </c>
       <c r="F21" s="9">
-        <f>IFERROR('Claim 05'!I45,"")</f>
+        <f>IFERROR('Claim 05'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8789,11 +8791,11 @@
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>IFERROR('Claim 06'!I44,"")</f>
+        <f>IFERROR('Claim 06'!D44,"")</f>
         <v/>
       </c>
       <c r="F22" s="9">
-        <f>IFERROR('Claim 06'!I45,"")</f>
+        <f>IFERROR('Claim 06'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8814,11 +8816,11 @@
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>IFERROR('Claim 07'!I44,"")</f>
+        <f>IFERROR('Claim 07'!D44,"")</f>
         <v/>
       </c>
       <c r="F23" s="9">
-        <f>IFERROR('Claim 07'!I45,"")</f>
+        <f>IFERROR('Claim 07'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8839,11 +8841,11 @@
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>IFERROR('Claim 08'!I44,"")</f>
+        <f>IFERROR('Claim 08'!D44,"")</f>
         <v/>
       </c>
       <c r="F24" s="9">
-        <f>IFERROR('Claim 08'!I45,"")</f>
+        <f>IFERROR('Claim 08'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8864,11 +8866,11 @@
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>IFERROR('Claim 09'!I44,"")</f>
+        <f>IFERROR('Claim 09'!D44,"")</f>
         <v/>
       </c>
       <c r="F25" s="9">
-        <f>IFERROR('Claim 09'!I45,"")</f>
+        <f>IFERROR('Claim 09'!D45,"")</f>
         <v/>
       </c>
     </row>
@@ -8889,11 +8891,11 @@
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>IFERROR('Claim 10'!I44,"")</f>
+        <f>IFERROR('Claim 10'!D44,"")</f>
         <v/>
       </c>
       <c r="F26" s="9">
-        <f>IFERROR('Claim 10'!I45,"")</f>
+        <f>IFERROR('Claim 10'!D45,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 'Date of audit' header field on row 7
Adds a new header row (A7 label 'Date of audit:', B7 yellow input,
YYYY-MM-DD format) to the Audit Checklist template and every Claim
01-10 tab so the auditor can record when they performed the review.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -420,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -710,6 +710,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1494,7 +1497,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -1850,7 +1860,6 @@
       <c r="E33" s="10" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
-    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
@@ -1986,7 +1995,6 @@
       </c>
       <c r="E42" s="14" t="inlineStr"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="44" customHeight="1">
       <c r="A44" s="38" t="inlineStr">
         <is>
@@ -2317,7 +2325,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -3022,7 +3037,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -3727,7 +3749,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -9179,7 +9208,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -9884,7 +9920,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -10589,7 +10632,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -11294,7 +11344,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -11999,7 +12056,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -12704,7 +12768,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -13409,7 +13480,14 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="52" t="n"/>
     </row>
-    <row r="7" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Date of audit:</t>
+        </is>
+      </c>
+      <c r="B7" s="109" t="n"/>
+    </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Defensively reset B5 to a clean Claim Number input
On the Audit Checklist template and every Claim 01-10 tab, B5 is now
guaranteed to be a plain yellow input with:
- No date number format (General)
- No data validation
- Empty value
- A5 label locked as 'Claim Number:'

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -420,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -711,6 +711,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1467,13 +1470,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -2295,13 +2298,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -3007,13 +3010,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -3719,13 +3722,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -9178,13 +9181,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -9890,13 +9893,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -10602,13 +10605,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -11314,13 +11317,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -12026,13 +12029,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -12738,13 +12741,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>
@@ -13450,13 +13453,13 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Claim Number:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="110" t="n"/>
       <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Auditor:</t>

</xml_diff>

<commit_message>
Fix Provider Progression chart series references
The chart on Quarterly Report was pulling row 12 as data — but row 12
is the header row (Provider / Jan / Feb...). That made the first series
try to plot 'Jan', 'Feb'... as compliance percentages, which Excel
either drew as zeros or silently skipped, leaving the chart looking
empty.

Rebuild the chart with min_row=13 so only the 5 provider data rows
(13-17) become series, and set the row 12 header as the category axis.
All data, progression-table formulas, and sample audit log rows are
untouched.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FQCsD1ZdbqSqbtLgYtoLBe
</commit_message>
<xml_diff>
--- a/docs/Clinical_Documentation_Audit_Simple.xlsx
+++ b/docs/Clinical_Documentation_Audit_Simple.xlsx
@@ -848,39 +848,6 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Quarterly Report'!B12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="7"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Quarterly Report'!$C$12:$N$12</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Quarterly Report'!$C$12:$N$12</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
               <f>'Quarterly Report'!B13</f>
             </strRef>
           </tx>
@@ -910,8 +877,8 @@
           </val>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="1"/>
+          <order val="1"/>
           <tx>
             <strRef>
               <f>'Quarterly Report'!B14</f>
@@ -943,8 +910,8 @@
           </val>
         </ser>
         <ser>
-          <idx val="3"/>
-          <order val="3"/>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <strRef>
               <f>'Quarterly Report'!B15</f>
@@ -976,8 +943,8 @@
           </val>
         </ser>
         <ser>
-          <idx val="4"/>
-          <order val="4"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'Quarterly Report'!B16</f>
@@ -1009,8 +976,8 @@
           </val>
         </ser>
         <ser>
-          <idx val="5"/>
-          <order val="5"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
               <f>'Quarterly Report'!B17</f>

</xml_diff>